<commit_message>
Ultimate Architecture Upgrades: Cross-Encoder, Latent Inference, Personalized Reasoning
</commit_message>
<xml_diff>
--- a/team_PJ2001_IND.xlsx
+++ b/team_PJ2001_IND.xlsx
@@ -441,1800 +441,1800 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0049978</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>21.2042</v>
+        <v>27.3466</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.6 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (71%).</t>
+          <t xml:space="preserve">16.9 yrs exp as AI Engineer. Built the document ingestion pipeline (chunking, embedding via OpenAI embeddings, storing in Pinecon... Highly responsive (72%). </t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0025882</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>19.8417</v>
+        <v>25.3442</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5.6 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (79%).</t>
+          <t>7.7 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (60%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0064331</t>
+          <t>CAND_0012957</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>19.3062</v>
+        <v>24.3258</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.2 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (74%).</t>
+          <t>4.9 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (67%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>19.0816</v>
+        <v>22.5275</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>16.2 years exp as Senior Applied Scientist (Stable tenure). High hybrid RRF score. Highly responsive (81%).</t>
+          <t>6.8 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (77%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0070525</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>19.0781</v>
+        <v>21.9631</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5.4 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (93%).</t>
+          <t xml:space="preserve">7.3 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (78%). </t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0002025</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>19.0445</v>
+        <v>21.8889</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.9 years exp as Senior AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (80%).</t>
+          <t>5.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (75%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0002344</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>18.1825</v>
+        <v>21.8364</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.7 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (83%).</t>
+          <t xml:space="preserve">4.6 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (76%). </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0077552</t>
+          <t>CAND_0061339</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>18.1727</v>
+        <v>21.1362</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.4 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (54%).</t>
+          <t xml:space="preserve">4.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (90%). </t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0042506</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>17.941</v>
+        <v>20.7428</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4.2 years exp as Search Engineer (Stable tenure). High hybrid RRF score. Highly responsive (48%).</t>
+          <t xml:space="preserve">14.1 yrs exp as Applied ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (87%). </t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0082086</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>17.8298</v>
+        <v>20.727</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>6.0 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (85%).</t>
+          <t>4.9 yrs exp as Machine Learning Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (79%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0060257</t>
+          <t>CAND_0030827</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>17.5143</v>
+        <v>20.6853</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5.8 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (56%).</t>
+          <t>5.4 yrs exp as Senior Data Scientist. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (52%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0065195</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>17.3458</v>
+        <v>20.4497</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>7.2 years exp as Senior Machine Learning Engineer (Stable tenure). High hybrid RRF score. Highly responsive (61%).</t>
+          <t>5.1 yrs exp as Search Engineer. Built the document ingestion pipeline (chunking, embedding via OpenAI embeddings, storing in Pinecon... Highly responsive (80%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0091534</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>17.1927</v>
+        <v>19.6154</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7.8 years exp as Senior AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (76%).</t>
+          <t xml:space="preserve">16.6 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (84%). </t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0064904</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>17.1587</v>
+        <v>18.5961</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>7.8 years exp as Senior NLP Engineer (Stable tenure). High hybrid RRF score. Highly responsive (89%).</t>
+          <t xml:space="preserve">4.9 yrs exp as AI Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (78%). </t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0060835</t>
+          <t>CAND_0022812</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>17.1463</v>
+        <v>18.075</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>6.6 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (32%).</t>
+          <t>4.5 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (79%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0009024</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>17.0496</v>
+        <v>17.1795</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4.6 years exp as AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (76%).</t>
+          <t xml:space="preserve">5.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (46%). </t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>17.0163</v>
+        <v>17.1625</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>7.3 years exp as AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (78%).</t>
+          <t>5.9 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0053591</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>16.9265</v>
+        <v>16.8219</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5.3 years exp as AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (81%).</t>
+          <t xml:space="preserve">6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). </t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0045027</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>16.7541</v>
+        <v>16.0632</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>8.6 years exp as Staff Machine Learning Engineer (Stable tenure). High hybrid RRF score. Highly responsive (83%).</t>
+          <t>3.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (80%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0002793</t>
+          <t>CAND_0082086</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>16.5645</v>
+        <v>15.8611</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>5.5 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (77%).</t>
+          <t xml:space="preserve">6.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (85%). </t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
+          <t>CAND_0060886</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>16.5249</v>
+        <v>15.8113</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>5.3 years exp as Senior Applied Scientist (Stable tenure). High hybrid RRF score. Highly responsive (55%).</t>
+          <t>4.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (38%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0082262</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>16.4521</v>
+        <v>15.5735</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>6.7 years exp as Lead AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (73%).</t>
+          <t>5.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (64%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0096104</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>16.2393</v>
+        <v>15.1946</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>7.0 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (33%).</t>
+          <t>5.2 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (47%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0074225</t>
+          <t>CAND_0076251</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>16.2338</v>
+        <v>15.0809</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>4.3 years exp as Machine Learning Engineer (Stable tenure). High hybrid RRF score. Highly responsive (91%).</t>
+          <t xml:space="preserve">7.6 yrs exp as Search Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (51%). </t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0091899</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>16.1111</v>
+        <v>14.5098</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>16.9 years exp as AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (72%).</t>
+          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (51%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0091348</t>
+          <t>CAND_0096104</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>15.9893</v>
+        <v>14.3709</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3.7 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (86%).</t>
+          <t>7.0 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (33%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0091229</t>
+          <t>CAND_0010408</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>15.9563</v>
+        <v>14.056</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>7.0 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (35%).</t>
+          <t>5.7 yrs exp as Junior ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (36%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0007411</t>
+          <t>CAND_0025923</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>15.7988</v>
+        <v>13.7933</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>8.0 years exp as Senior Machine Learning Engineer (Stable tenure). High hybrid RRF score. Highly responsive (12%).</t>
+          <t>5.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (84%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0082913</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>15.7988</v>
+        <v>13.792</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>5.5 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (73%).</t>
+          <t xml:space="preserve">6.9 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (65%). </t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0062707</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>15.5962</v>
+        <v>13.6763</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>8.0 years exp as Recommendation Systems Engineer (Stable tenure). High hybrid RRF score. Highly responsive (77%).</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0052328</t>
+          <t>CAND_0058412</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>15.5951</v>
+        <v>13.5997</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>6.5 years exp as Recommendation Systems Engineer (Stable tenure). High hybrid RRF score. Highly responsive (79%).</t>
+          <t xml:space="preserve">6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (43%). </t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0018549</t>
+          <t>CAND_0068892</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>15.5818</v>
+        <v>13.5038</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>6.8 years exp as Recommendation Systems Engineer (Stable tenure). High hybrid RRF score. Highly responsive (73%).</t>
+          <t>4.7 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (51%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0059795</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>15.5583</v>
+        <v>13.3581</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>8.9 years exp as Senior NLP Engineer (Stable tenure). High hybrid RRF score. Highly responsive (78%).</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (75%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0018961</t>
+          <t>CAND_0074325</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>15.2965</v>
+        <v>13.1659</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>5.0 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (26%).</t>
+          <t xml:space="preserve">3.9 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (47%). </t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0060886</t>
+          <t>CAND_0061156</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>15.1735</v>
+        <v>13.081</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>4.6 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (38%).</t>
+          <t xml:space="preserve">6.0 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (39%). </t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0017960</t>
+          <t>CAND_0009516</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>15.1455</v>
+        <v>13.0748</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>7.7 years exp as Recommendation Systems Engineer (Stable tenure). High hybrid RRF score. Highly responsive (72%).</t>
+          <t>6.9 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (34%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0005269</t>
+          <t>CAND_0077552</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>15.1343</v>
+        <v>13.0099</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>6.1 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (28%).</t>
+          <t>3.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0088526</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>15.0896</v>
+        <v>12.9754</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>7.7 years exp as AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (60%).</t>
+          <t xml:space="preserve">4.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). </t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0091534</t>
+          <t>CAND_0091348</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>15.0585</v>
+        <v>12.8321</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>16.6 years exp as AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (84%).</t>
+          <t>3.7 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (86%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0068892</t>
+          <t>CAND_0060257</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>14.9373</v>
+        <v>12.7828</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>4.7 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (51%).</t>
+          <t xml:space="preserve">5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%). </t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0015097</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>14.8718</v>
+        <v>12.4961</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>6.9 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (65%).</t>
+          <t xml:space="preserve">6.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (69%). </t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0061156</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>14.8693</v>
+        <v>12.4049</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>6.0 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (39%).</t>
+          <t xml:space="preserve">6.8 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%). </t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0042029</t>
+          <t>CAND_0078810</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>14.853</v>
+        <v>12.3073</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>6.5 years exp as Senior Data Scientist (Stable tenure). High hybrid RRF score. Highly responsive (67%).</t>
+          <t xml:space="preserve">6.9 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). </t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0072032</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>14.7763</v>
+        <v>12.2858</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>7.0 years exp as Staff Machine Learning Engineer (Stable tenure). High hybrid RRF score. Highly responsive (95%).</t>
+          <t xml:space="preserve">6.1 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (38%). </t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0015097</t>
+          <t>CAND_0004402</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>14.6819</v>
+        <v>12.2244</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>6.0 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (69%).</t>
+          <t xml:space="preserve">6.0 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). </t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0058152</t>
+          <t>CAND_0013665</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>14.6158</v>
+        <v>12.1053</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3.6 years exp as Data Scientist (Stable tenure). High hybrid RRF score. Highly responsive (85%).</t>
+          <t>5.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0037566</t>
+          <t>CAND_0018961</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>14.563</v>
+        <v>11.999</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>6.9 years exp as Machine Learning Engineer (Stable tenure). High hybrid RRF score. Highly responsive (50%).</t>
+          <t xml:space="preserve">5.0 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (26%). </t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0079688</t>
+          <t>CAND_0005269</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>14.5618</v>
+        <v>11.9684</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>3.3 years exp as Senior Software Engineer (ML) (Stable tenure). High hybrid RRF score. Highly responsive (69%).</t>
+          <t>6.1 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0010541</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>14.5526</v>
+        <v>11.9621</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>6.1 years exp as Senior Machine Learning Engineer (Stable tenure). High hybrid RRF score. Highly responsive (88%).</t>
+          <t>6.2 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (59%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0008628</t>
+          <t>CAND_0073007</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>14.5477</v>
+        <v>11.9401</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3.2 years exp as AI Specialist (High mobility). High hybrid RRF score. Highly responsive (54%).</t>
+          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0029439</t>
+          <t>CAND_0046313</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>14.5425</v>
+        <v>11.8775</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>6.4 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (60%).</t>
+          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (45%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0064326</t>
+          <t>CAND_0007008</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>14.4243</v>
+        <v>11.8503</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>7.6 years exp as Search Engineer (Stable tenure). High hybrid RRF score. Highly responsive (94%).</t>
+          <t>3.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (66%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0024878</t>
+          <t>CAND_0066309</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>14.4235</v>
+        <v>11.833</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>5.7 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (84%).</t>
+          <t xml:space="preserve">5.3 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%). </t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0098780</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>14.4048</v>
+        <v>11.8308</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>5.9 years exp as AI Research Engineer (Stable tenure). High hybrid RRF score. Highly responsive (56%).</t>
+          <t xml:space="preserve">6.1 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (81%). </t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0079550</t>
+          <t>CAND_0008218</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>14.3907</v>
+        <v>11.6889</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>3.9 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (88%).</t>
+          <t xml:space="preserve">7.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (39%). </t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0024947</t>
+          <t>CAND_0003609</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>14.3743</v>
+        <v>11.5924</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>6.1 years exp as AI Research Engineer (Stable tenure). High hybrid RRF score. Highly responsive (79%).</t>
+          <t>6.1 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (50%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0030031</t>
+          <t>CAND_0024947</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>14.1369</v>
+        <v>11.5669</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>5.7 years exp as AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (94%).</t>
+          <t xml:space="preserve">6.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). </t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0059017</t>
+          <t>CAND_0075502</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>13.8228</v>
+        <v>11.3895</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>6.8 years exp as AI Research Engineer (Stable tenure). High hybrid RRF score. Highly responsive (75%).</t>
+          <t xml:space="preserve">3.3 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). </t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0043312</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>13.7971</v>
+        <v>11.3713</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>8.6 years exp as Lead AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (11%).</t>
+          <t xml:space="preserve">4.2 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (73%). </t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>13.6788</v>
+        <v>11.3636</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>8.1 years exp as Senior Machine Learning Engineer (Stable tenure). High hybrid RRF score. Highly responsive (87%).</t>
+          <t>5.2 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0004402</t>
+          <t>CAND_0002344</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>13.6321</v>
+        <v>11.3491</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>6.0 years exp as AI Research Engineer (Stable tenure). High hybrid RRF score. Highly responsive (83%).</t>
+          <t xml:space="preserve">4.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (83%). </t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0074325</t>
+          <t>CAND_0026942</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>13.6319</v>
+        <v>11.3124</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>3.9 years exp as AI Research Engineer (Stable tenure). High hybrid RRF score. Highly responsive (47%).</t>
+          <t>6.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0072032</t>
+          <t>CAND_0074648</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>13.4052</v>
+        <v>11.3074</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>6.1 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (38%).</t>
+          <t xml:space="preserve">4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (82%). </t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0045250</t>
+          <t>CAND_0088878</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>13.3268</v>
+        <v>11.2084</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>6.6 years exp as Applied ML Engineer (Stable tenure). High hybrid RRF score. Highly responsive (74%).</t>
+          <t>4.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (31%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0065195</t>
+          <t>CAND_0077498</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>13.2559</v>
+        <v>11.1701</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>5.1 years exp as Search Engineer (Stable tenure). High hybrid RRF score. Highly responsive (80%).</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (89%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0009200</t>
+          <t>CAND_0079550</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>13.2356</v>
+        <v>10.9318</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>5.7 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (32%).</t>
+          <t>3.9 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (88%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0073007</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>13.1131</v>
+        <v>10.8838</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>5.8 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (83%).</t>
+          <t xml:space="preserve">7.1 yrs exp as Applied ML Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (61%). </t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0037944</t>
+          <t>CAND_0060315</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>13.0772</v>
+        <v>10.837</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>4.9 years exp as Senior Data Scientist (Stable tenure). High hybrid RRF score. Highly responsive (42%).</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (63%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0079176</t>
+          <t>CAND_0064331</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>13.0476</v>
+        <v>10.7195</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>5.3 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (73%).</t>
+          <t xml:space="preserve">4.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (74%). </t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0033861</t>
+          <t>CAND_0077956</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>12.9261</v>
+        <v>10.6404</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>8.0 years exp as Senior NLP Engineer (Stable tenure). High hybrid RRF score. Highly responsive (16%).</t>
+          <t>6.4 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (88%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0024147</t>
+          <t>CAND_0025882</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>12.9145</v>
+        <v>10.5707</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>5.9 years exp as ML Engineer (Stable tenure). High hybrid RRF score. Highly responsive (84%).</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0006418</t>
+          <t>CAND_0061175</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>12.8774</v>
+        <v>10.4232</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>5.7 years exp as Machine Learning Engineer (Stable tenure). High hybrid RRF score. Highly responsive (92%).</t>
+          <t xml:space="preserve">6.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%). </t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0014063</t>
+          <t>CAND_0065139</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>12.8463</v>
+        <v>10.4123</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>5.4 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (69%).</t>
+          <t>5.2 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (82%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0016657</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>12.8414</v>
+        <v>10.3707</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>6.8 years exp as Applied ML Engineer (Stable tenure). High hybrid RRF score. Highly responsive (41%).</t>
+          <t>5.3 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (52%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0075249</t>
+          <t>CAND_0002793</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>12.7866</v>
+        <v>10.3484</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>6.2 years exp as Applied ML Engineer (Stable tenure). High hybrid RRF score. Highly responsive (82%).</t>
+          <t xml:space="preserve">5.5 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (77%). </t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0052498</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>12.7452</v>
+        <v>10.2909</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>6.9 years exp as AI Engineer (Stable tenure). High hybrid RRF score. Highly responsive (81%).</t>
+          <t>4.7 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (28%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0098952</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>12.6587</v>
+        <v>10.2645</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>5.2 years exp as ML Engineer (Stable tenure). High hybrid RRF score. Highly responsive (48%).</t>
+          <t>5.5 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (66%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0019845</t>
+          <t>CAND_0069638</t>
         </is>
       </c>
       <c r="B79" t="n">
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>12.5688</v>
+        <v>10.0109</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>3.4 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (78%).</t>
+          <t>6.2 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (64%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0080315</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>12.5423</v>
+        <v>10.0035</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>6.1 years exp as Junior ML Engineer (Stable tenure). High hybrid RRF score. Highly responsive (81%).</t>
+          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0076412</t>
+          <t>CAND_0058152</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>12.5131</v>
+        <v>9.8194</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>5.8 years exp as AI Research Engineer (Stable tenure). High hybrid RRF score. Highly responsive (54%).</t>
+          <t xml:space="preserve">3.6 yrs exp as Data Scientist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (85%). </t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0013122</t>
+          <t>CAND_0016170</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>12.4904</v>
+        <v>9.7112</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>4.3 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (56%).</t>
+          <t xml:space="preserve">6.8 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (52%). </t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0012632</t>
+          <t>CAND_0019845</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>12.4876</v>
+        <v>9.6617</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>6.0 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (53%).</t>
+          <t>3.4 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (78%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0041611</t>
+          <t>CAND_0081480</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>12.4434</v>
+        <v>9.6502</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>6.4 years exp as Staff Machine Learning Engineer (Stable tenure). High hybrid RRF score. Highly responsive (7%).</t>
+          <t xml:space="preserve">5.6 yrs exp as Computer Vision Engineer. Strong semantic alignment with AI system requirements. Highly responsive (85%). </t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0098952</t>
+          <t>CAND_0008628</t>
         </is>
       </c>
       <c r="B85" t="n">
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>12.3434</v>
+        <v>9.595000000000001</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>5.5 years exp as AI Research Engineer (Stable tenure). High hybrid RRF score. Highly responsive (66%).</t>
+          <t>3.2 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0012957</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>12.2768</v>
+        <v>9.579800000000001</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>4.9 years exp as Search Engineer (Stable tenure). High hybrid RRF score. Highly responsive (67%).</t>
+          <t xml:space="preserve">5.8 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (57%). </t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0030953</t>
+          <t>CAND_0070525</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>12.2485</v>
+        <v>9.551</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>7.8 years exp as Search Engineer (Stable tenure). High hybrid RRF score. Highly responsive (63%).</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (93%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0061265</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B88" t="n">
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>12.1922</v>
+        <v>9.533099999999999</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>6.6 years exp as Recommendation Systems Engineer (Stable tenure). High hybrid RRF score. Highly responsive (94%).</t>
+          <t xml:space="preserve">5.0 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). </t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0010541</t>
+          <t>CAND_0080597</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>12.1841</v>
+        <v>9.297499999999999</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>6.2 years exp as AI Research Engineer (Stable tenure). High hybrid RRF score. Highly responsive (59%).</t>
+          <t>4.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (33%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0084161</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>12.1501</v>
+        <v>9.282500000000001</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>5.0 years exp as ML Engineer (Stable tenure). High hybrid RRF score. Highly responsive (71%).</t>
+          <t>3.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (77%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0092568</t>
+          <t>CAND_0059520</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>12.1381</v>
+        <v>9.2661</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>5.7 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (39%).</t>
+          <t>4.3 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (36%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0052682</t>
+          <t>CAND_0091229</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>12.129</v>
+        <v>9.258699999999999</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>6.6 years exp as NLP Engineer (Stable tenure). High hybrid RRF score. Highly responsive (88%).</t>
+          <t xml:space="preserve">7.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (35%). </t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0002426</t>
+          <t>CAND_0091890</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>12.0855</v>
+        <v>9.1813</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>3.3 years exp as Data Scientist (Stable tenure). High hybrid RRF score. Highly responsive (80%).</t>
+          <t xml:space="preserve">4.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (49%). </t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0078002</t>
+          <t>CAND_0060835</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>12.0315</v>
+        <v>9.0395</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>6.3 years exp as Machine Learning Engineer (Stable tenure). High hybrid RRF score. Highly responsive (86%).</t>
+          <t xml:space="preserve">6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (32%). </t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0007009</t>
+          <t>CAND_0031306</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>11.9926</v>
+        <v>8.9565</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>7.9 years exp as Recommendation Systems Engineer (Stable tenure). High hybrid RRF score. Highly responsive (62%).</t>
+          <t>3.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0077881</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>11.9876</v>
+        <v>8.903600000000001</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>6.7 years exp as AI Research Engineer (Stable tenure). High hybrid RRF score. Highly responsive (48%).</t>
+          <t xml:space="preserve">4.6 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (30%). </t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0091580</t>
+          <t>CAND_0084681</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>11.9803</v>
+        <v>8.886200000000001</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>5.5 years exp as Data Scientist (Stable tenure). High hybrid RRF score. Highly responsive (25%).</t>
+          <t xml:space="preserve">3.5 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (67%). </t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0014715</t>
+          <t>CAND_0013122</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>11.9336</v>
+        <v>8.880599999999999</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>4.2 years exp as AI Specialist (Stable tenure). High hybrid RRF score. Highly responsive (27%).</t>
+          <t>4.3 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0042359</t>
+          <t>CAND_0012632</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>11.9188</v>
+        <v>8.870100000000001</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>6.9 years exp as Data Scientist (Stable tenure). High hybrid RRF score. Highly responsive (76%).</t>
+          <t>6.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (53%). Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0053695</t>
+          <t>CAND_0077261</t>
         </is>
       </c>
       <c r="B100" t="n">
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>11.8756</v>
+        <v>8.8691</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>5.8 years exp as Recommendation Systems Engineer (Stable tenure). High hybrid RRF score. Highly responsive (60%).</t>
+          <t xml:space="preserve">5.7 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (81%). </t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0069905</t>
+          <t>CAND_0091745</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>11.8361</v>
+        <v>8.8184</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>6.6 years exp as Applied ML Engineer (Stable tenure). High hybrid RRF score. Highly responsive (78%).</t>
+          <t xml:space="preserve">5.9 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (53%). </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The Ultimate Masterpiece: Dashboard UI Overhaul, Promotion Detector, Skill Decay
</commit_message>
<xml_diff>
--- a/team_PJ2001_IND.xlsx
+++ b/team_PJ2001_IND.xlsx
@@ -441,36 +441,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0044222</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>27.3466</v>
+        <v>27.0516</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">16.9 yrs exp as AI Engineer. Built the document ingestion pipeline (chunking, embedding via OpenAI embeddings, storing in Pinecon... Highly responsive (72%). </t>
+          <t>7.7 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (60%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>25.3442</v>
+        <v>25.4856</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7.7 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (60%). Lifelong Learner.</t>
+          <t>16.9 yrs exp as AI Engineer. Built the document ingestion pipeline (chunking, embedding via OpenAI embeddings, storing in Pinecon... Highly responsive (72%).</t>
         </is>
       </c>
     </row>
@@ -484,11 +484,11 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>24.3258</v>
+        <v>23.7626</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (67%). Lifelong Learner.</t>
+          <t>4.9 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (67%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
@@ -502,11 +502,11 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>22.5275</v>
+        <v>22.6142</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.8 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (77%). Lifelong Learner.</t>
+          <t>6.8 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (77%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
@@ -520,47 +520,47 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>21.9631</v>
+        <v>22.2456</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.3 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (78%). </t>
+          <t>7.3 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (78%).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>21.8889</v>
+        <v>22.021</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (75%). Lifelong Learner.</t>
+          <t>4.6 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (76%).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>21.8364</v>
+        <v>21.2042</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.6 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (76%). </t>
+          <t>14.1 yrs exp as Applied ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (87%).</t>
         </is>
       </c>
     </row>
@@ -574,209 +574,209 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>21.1362</v>
+        <v>20.6349</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (90%). </t>
+          <t>4.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (90%).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>20.7428</v>
+        <v>20.5114</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">14.1 yrs exp as Applied ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (87%). </t>
+          <t>5.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (75%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0030827</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>20.727</v>
+        <v>20.4751</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as Machine Learning Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (79%). Lifelong Learner.</t>
+          <t>5.4 yrs exp as Senior Data Scientist. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (52%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0030827</t>
+          <t>CAND_0091534</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>20.6853</v>
+        <v>20.3934</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Data Scientist. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (52%). Lifelong Learner.</t>
+          <t>16.6 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (84%).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0065195</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>20.4497</v>
+        <v>20.2546</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5.1 yrs exp as Search Engineer. Built the document ingestion pipeline (chunking, embedding via OpenAI embeddings, storing in Pinecon... Highly responsive (80%). Lifelong Learner.</t>
+          <t>4.9 yrs exp as Machine Learning Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (79%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0091534</t>
+          <t>CAND_0064904</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>19.6154</v>
+        <v>18.8519</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">16.6 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (84%). </t>
+          <t>4.9 yrs exp as AI Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (78%).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
+          <t>CAND_0009024</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>18.5961</v>
+        <v>17.0339</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.9 yrs exp as AI Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (78%). </t>
+          <t>5.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (46%).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0022812</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>18.075</v>
+        <v>16.5409</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>4.5 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (79%). Lifelong Learner.</t>
+          <t>5.9 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0009024</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>17.1795</v>
+        <v>16.3944</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (46%). </t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0024620</t>
+          <t>CAND_0060886</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>17.1625</v>
+        <v>16.0829</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>5.9 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%). Lifelong Learner.</t>
+          <t>4.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (38%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0049978</t>
+          <t>CAND_0045027</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>16.8219</v>
+        <v>16.0088</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). </t>
+          <t>3.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (80%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0045027</t>
+          <t>CAND_0022812</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>16.0632</v>
+        <v>15.9683</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>3.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (80%). Lifelong Learner.</t>
+          <t>4.5 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (79%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
@@ -790,29 +790,29 @@
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>15.8611</v>
+        <v>15.9508</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (85%). </t>
+          <t>6.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (85%).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0060886</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>15.8113</v>
+        <v>15.5263</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (38%). Lifelong Learner.</t>
+          <t>5.2 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (47%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
@@ -826,155 +826,155 @@
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>15.5735</v>
+        <v>15.0779</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>5.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (64%). Lifelong Learner.</t>
+          <t>5.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (64%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0024466</t>
+          <t>CAND_0076251</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>15.1946</v>
+        <v>15.0083</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (47%). Lifelong Learner.</t>
+          <t>7.6 yrs exp as Search Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (51%).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0076251</t>
+          <t>CAND_0091899</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>15.0809</v>
+        <v>14.4385</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.6 yrs exp as Search Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (51%). </t>
+          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (51%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0091899</t>
+          <t>CAND_0068892</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>14.5098</v>
+        <v>14.1872</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (51%). Lifelong Learner.</t>
+          <t>4.7 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (51%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0096104</t>
+          <t>CAND_0025923</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>14.3709</v>
+        <v>14.0658</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>7.0 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (33%). Lifelong Learner.</t>
+          <t>5.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (84%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0010408</t>
+          <t>CAND_0060257</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>14.056</v>
+        <v>14.0019</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5.7 yrs exp as Junior ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (36%). Lifelong Learner.</t>
+          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0025923</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>13.7933</v>
+        <v>13.8787</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (84%). Lifelong Learner.</t>
+          <t>6.9 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (65%).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0010408</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>13.792</v>
+        <v>13.8609</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.9 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (65%). </t>
+          <t>5.7 yrs exp as Junior ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (36%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0062707</t>
+          <t>CAND_0096104</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>13.6763</v>
+        <v>13.5991</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). Lifelong Learner.</t>
+          <t>7.0 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (33%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
@@ -988,29 +988,29 @@
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>13.5997</v>
+        <v>13.5407</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (43%). </t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (43%).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0068892</t>
+          <t>CAND_0062707</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>13.5038</v>
+        <v>13.2556</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (51%). Lifelong Learner.</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
@@ -1024,29 +1024,29 @@
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>13.3581</v>
+        <v>13.2344</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (75%). Lifelong Learner.</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (75%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0074325</t>
+          <t>CAND_0088526</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>13.1659</v>
+        <v>13.1835</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.9 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (47%). </t>
+          <t>4.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). Fast-track promotions.</t>
         </is>
       </c>
     </row>
@@ -1060,29 +1060,29 @@
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>13.081</v>
+        <v>13.1417</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.0 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (39%). </t>
+          <t>6.0 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (39%).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0009516</t>
+          <t>CAND_0015097</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>13.0748</v>
+        <v>12.8625</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>6.9 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (34%). Lifelong Learner.</t>
+          <t>6.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (69%).</t>
         </is>
       </c>
     </row>
@@ -1096,605 +1096,605 @@
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>13.0099</v>
+        <v>12.6173</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%). Lifelong Learner.</t>
+          <t>3.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0088526</t>
+          <t>CAND_0091348</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>12.9754</v>
+        <v>12.563</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). </t>
+          <t>3.7 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (86%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0091348</t>
+          <t>CAND_0013665</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>12.8321</v>
+        <v>12.2595</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (86%). Lifelong Learner.</t>
+          <t>5.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0060257</t>
+          <t>CAND_0078810</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>12.7828</v>
+        <v>12.2595</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%). </t>
+          <t>6.9 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0015097</t>
+          <t>CAND_0010541</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>12.4961</v>
+        <v>12.229</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (69%). </t>
+          <t>6.2 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (59%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0005269</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>12.4049</v>
+        <v>12.21</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.8 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%). </t>
+          <t>6.1 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0078810</t>
+          <t>CAND_0043312</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>12.3073</v>
+        <v>12.2076</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.9 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). </t>
+          <t>4.2 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (73%).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0072032</t>
+          <t>CAND_0007008</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>12.2858</v>
+        <v>12.1736</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.1 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (38%). </t>
+          <t>3.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (66%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0004402</t>
+          <t>CAND_0046313</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>12.2244</v>
+        <v>12.0981</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.0 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). </t>
+          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (45%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0013665</t>
+          <t>CAND_0074325</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>12.1053</v>
+        <v>12.0855</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). Lifelong Learner.</t>
+          <t>3.9 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (47%).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0018961</t>
+          <t>CAND_0009516</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>11.999</v>
+        <v>12.0486</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.0 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (26%). </t>
+          <t>6.9 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (34%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0005269</t>
+          <t>CAND_0074648</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>11.9684</v>
+        <v>12.0098</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%). Lifelong Learner.</t>
+          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (82%).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0010541</t>
+          <t>CAND_0003609</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>11.9621</v>
+        <v>11.9048</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>6.2 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (59%). Lifelong Learner.</t>
+          <t>6.1 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (50%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0073007</t>
+          <t>CAND_0079688</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>11.9401</v>
+        <v>11.7606</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). Lifelong Learner.</t>
+          <t>3.3 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (69%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0046313</t>
+          <t>CAND_0077956</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>11.8775</v>
+        <v>11.6738</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (45%). Lifelong Learner.</t>
+          <t>6.4 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (88%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0007008</t>
+          <t>CAND_0089249</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>11.8503</v>
+        <v>11.5768</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (66%). Lifelong Learner.</t>
+          <t>3.1 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (47%).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0066309</t>
+          <t>CAND_0004402</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>11.833</v>
+        <v>11.5596</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.3 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%). </t>
+          <t>6.0 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%).</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0018961</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>11.8308</v>
+        <v>11.4328</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.1 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (81%). </t>
+          <t>5.0 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (26%).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0008218</t>
+          <t>CAND_0072032</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>11.6889</v>
+        <v>11.3558</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (39%). </t>
+          <t>6.1 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (38%).</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0003609</t>
+          <t>CAND_0073007</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>11.5924</v>
+        <v>11.3265</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (50%). Lifelong Learner.</t>
+          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0024947</t>
+          <t>CAND_0026942</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>11.5669</v>
+        <v>11.3171</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). </t>
+          <t>6.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0075502</t>
+          <t>CAND_0082913</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>11.3895</v>
+        <v>11.2736</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.3 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). </t>
+          <t>5.5 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%).</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0043312</t>
+          <t>CAND_0088878</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>11.3713</v>
+        <v>11.2392</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.2 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (73%). </t>
+          <t>4.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (31%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0008218</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>11.3636</v>
+        <v>11.1902</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%). Lifelong Learner.</t>
+          <t>7.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (39%).</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0002344</t>
+          <t>CAND_0077498</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>11.3491</v>
+        <v>11.0874</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (83%). </t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (89%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0026942</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>11.3124</v>
+        <v>11.0303</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). Lifelong Learner.</t>
+          <t>6.8 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0074648</t>
+          <t>CAND_0024947</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>11.3074</v>
+        <v>11.0223</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (82%). </t>
+          <t>6.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%).</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0088878</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>11.2084</v>
+        <v>11.0203</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>4.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (31%). Lifelong Learner.</t>
+          <t>6.1 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (81%).</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0077498</t>
+          <t>CAND_0075502</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>11.1701</v>
+        <v>10.9718</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (89%). Lifelong Learner.</t>
+          <t>3.3 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%).</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0079550</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>10.9318</v>
+        <v>10.9629</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (88%). Lifelong Learner.</t>
+          <t>5.2 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0002344</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>10.8838</v>
+        <v>10.9202</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.1 yrs exp as Applied ML Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (61%). </t>
+          <t>4.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (83%).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0060315</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>10.837</v>
+        <v>10.8376</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (63%). Lifelong Learner.</t>
+          <t>7.1 yrs exp as Applied ML Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (61%).</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0064331</t>
+          <t>CAND_0079550</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>10.7195</v>
+        <v>10.7789</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (74%). </t>
+          <t>3.9 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (88%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0077956</t>
+          <t>CAND_0060315</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>10.6404</v>
+        <v>10.7168</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>6.4 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (88%). Lifelong Learner.</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (63%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
@@ -1708,65 +1708,65 @@
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>10.5707</v>
+        <v>10.6615</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). Lifelong Learner.</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0098952</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>10.4232</v>
+        <v>10.6221</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%). </t>
+          <t>5.5 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (66%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0065139</t>
+          <t>CAND_0012988</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>10.4123</v>
+        <v>10.6132</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (82%). Lifelong Learner.</t>
+          <t>4.3 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%).</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0016657</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>10.3707</v>
+        <v>10.4847</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>5.3 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (52%). Lifelong Learner.</t>
+          <t>5.0 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%).</t>
         </is>
       </c>
     </row>
@@ -1780,461 +1780,461 @@
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>10.3484</v>
+        <v>10.3095</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.5 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (77%). </t>
+          <t>5.5 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (77%).</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0052498</t>
+          <t>CAND_0016657</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>10.2909</v>
+        <v>10.2182</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (28%). Lifelong Learner.</t>
+          <t>5.3 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (52%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0098952</t>
+          <t>CAND_0070525</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>10.2645</v>
+        <v>9.8941</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>5.5 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (66%). Lifelong Learner.</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (93%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0069638</t>
+          <t>CAND_0061175</t>
         </is>
       </c>
       <c r="B79" t="n">
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>10.0109</v>
+        <v>9.8934</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>6.2 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (64%). Lifelong Learner.</t>
+          <t>6.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%).</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0080315</t>
+          <t>CAND_0065139</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>10.0035</v>
+        <v>9.869199999999999</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%). Lifelong Learner.</t>
+          <t>5.2 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (82%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0058152</t>
+          <t>CAND_0064331</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>9.8194</v>
+        <v>9.8558</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.6 yrs exp as Data Scientist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (85%). </t>
+          <t>4.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (74%).</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0016170</t>
+          <t>CAND_0080315</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>9.7112</v>
+        <v>9.793799999999999</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.8 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (52%). </t>
+          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0019845</t>
+          <t>CAND_0009200</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>9.6617</v>
+        <v>9.715299999999999</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>3.4 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (78%). Lifelong Learner.</t>
+          <t>5.7 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (32%).</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0081480</t>
+          <t>CAND_0069638</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>9.6502</v>
+        <v>9.6838</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.6 yrs exp as Computer Vision Engineer. Strong semantic alignment with AI system requirements. Highly responsive (85%). </t>
+          <t>6.2 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (64%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0008628</t>
+          <t>CAND_0014063</t>
         </is>
       </c>
       <c r="B85" t="n">
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>9.595000000000001</v>
+        <v>9.588699999999999</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>3.2 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%). Lifelong Learner.</t>
+          <t>5.4 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (69%).</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0081480</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>9.579800000000001</v>
+        <v>9.5494</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.8 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (57%). </t>
+          <t>5.6 yrs exp as Computer Vision Engineer. Strong semantic alignment with AI system requirements. Highly responsive (85%).</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0070525</t>
+          <t>CAND_0091890</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>9.551</v>
+        <v>9.4201</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (93%). Lifelong Learner.</t>
+          <t>4.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (49%).</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0084161</t>
         </is>
       </c>
       <c r="B88" t="n">
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>9.533099999999999</v>
+        <v>9.351100000000001</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.0 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). </t>
+          <t>3.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (77%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0080597</t>
+          <t>CAND_0060835</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>9.297499999999999</v>
+        <v>9.2898</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>4.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (33%). Lifelong Learner.</t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (32%).</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0084161</t>
+          <t>CAND_0077881</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>9.282500000000001</v>
+        <v>9.2624</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (77%). Lifelong Learner.</t>
+          <t>4.6 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (30%).</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0059520</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>9.2661</v>
+        <v>9.238899999999999</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>4.3 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (36%). Lifelong Learner.</t>
+          <t>5.8 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (57%).</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0091229</t>
+          <t>CAND_0031306</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>9.258699999999999</v>
+        <v>9.235900000000001</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (35%). </t>
+          <t>3.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0091890</t>
+          <t>CAND_0091745</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>9.1813</v>
+        <v>9.208600000000001</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (49%). </t>
+          <t>5.9 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (53%).</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0060835</t>
+          <t>CAND_0072721</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>9.0395</v>
+        <v>9.2029</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (32%). </t>
+          <t>3.7 yrs exp as Data Scientist. Strong semantic alignment with AI system requirements. Highly responsive (53%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0031306</t>
+          <t>CAND_0056584</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>8.9565</v>
+        <v>9.1015</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>3.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). Lifelong Learner.</t>
+          <t>3.5 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (69%).</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0077881</t>
+          <t>CAND_0008628</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>8.903600000000001</v>
+        <v>9.0868</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.6 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (30%). </t>
+          <t>3.2 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0084681</t>
+          <t>CAND_0080597</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>8.886200000000001</v>
+        <v>9.085000000000001</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.5 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (67%). </t>
+          <t>4.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (33%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0013122</t>
+          <t>CAND_0052498</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>8.880599999999999</v>
+        <v>9.0349</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>4.3 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%). Lifelong Learner.</t>
+          <t>4.7 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (28%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0012632</t>
+          <t>CAND_0091229</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>8.870100000000001</v>
+        <v>8.936500000000001</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (53%). Lifelong Learner.</t>
+          <t>7.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (35%).</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0077261</t>
+          <t>CAND_0059520</t>
         </is>
       </c>
       <c r="B100" t="n">
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>8.8691</v>
+        <v>8.930999999999999</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.7 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (81%). </t>
+          <t>4.3 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (36%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0091745</t>
+          <t>CAND_0012632</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>8.8184</v>
+        <v>8.8279</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.9 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (53%). </t>
+          <t>6.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (53%).  Lifelong Learner.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The Unthinkable Tier: Dunning-Kruger Filter, Elite Alumni Gravity, and X-Ray UI Dashboard
</commit_message>
<xml_diff>
--- a/team_PJ2001_IND.xlsx
+++ b/team_PJ2001_IND.xlsx
@@ -448,11 +448,11 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>27.0516</v>
+        <v>26.4706</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7.7 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (60%).  Lifelong Learner.</t>
+          <t>7.7 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (60%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
@@ -466,155 +466,155 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>25.4856</v>
+        <v>25.9109</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>16.9 yrs exp as AI Engineer. Built the document ingestion pipeline (chunking, embedding via OpenAI embeddings, storing in Pinecon... Highly responsive (72%).</t>
+          <t>16.9 yrs exp as AI Engineer. Built the document ingestion pipeline (chunking, embedding via OpenAI embeddings, storing in Pinecon... Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0012957</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>23.7626</v>
+        <v>23.4074</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (67%).  Lifelong Learner.</t>
+          <t>7.3 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0012957</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>22.6142</v>
+        <v>23.3754</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6.8 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (77%).  Lifelong Learner.</t>
+          <t>4.9 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (67%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>22.2456</v>
+        <v>21.8629</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.3 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (78%).</t>
+          <t>6.8 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (77%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>22.021</v>
+        <v>21.4646</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (76%).</t>
+          <t>5.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (75%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>21.2042</v>
+        <v>21.3721</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>14.1 yrs exp as Applied ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (87%).</t>
+          <t>4.9 yrs exp as Machine Learning Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0061339</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>20.6349</v>
+        <v>21.1153</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>4.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (90%).</t>
+          <t>14.1 yrs exp as Applied ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (87%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>20.5114</v>
+        <v>21.0775</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (75%).  Lifelong Learner.</t>
+          <t>4.6 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (76%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0030827</t>
+          <t>CAND_0061339</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>20.4751</v>
+        <v>20.9492</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Data Scientist. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (52%).  Lifelong Learner.</t>
+          <t>4.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (90%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
@@ -628,299 +628,299 @@
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>20.3934</v>
+        <v>20.6699</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>16.6 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (84%).</t>
+          <t>16.6 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0030827</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>20.2546</v>
+        <v>20.6129</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as Machine Learning Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (79%).  Lifelong Learner.</t>
+          <t>5.4 yrs exp as Senior Data Scientist. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (52%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
+          <t>CAND_0065195</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>18.8519</v>
+        <v>20.5058</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as AI Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (78%).</t>
+          <t>5.1 yrs exp as Search Engineer. Built the document ingestion pipeline (chunking, embedding via OpenAI embeddings, storing in Pinecon... Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0009024</t>
+          <t>CAND_0064904</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>17.0339</v>
+        <v>18.8519</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (46%).</t>
+          <t>4.9 yrs exp as AI Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0024620</t>
+          <t>CAND_0009024</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>16.5409</v>
+        <v>18.0062</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5.9 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%).  Lifelong Learner.</t>
+          <t>5.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (46%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0049978</t>
+          <t>CAND_0024620</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>16.3944</v>
+        <v>16.3938</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%).</t>
+          <t>5.9 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0060886</t>
+          <t>CAND_0022812</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>16.0829</v>
+        <v>16.0565</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (38%).  Lifelong Learner.</t>
+          <t>4.5 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0045027</t>
+          <t>CAND_0060886</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>16.0088</v>
+        <v>15.8784</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (80%).  Lifelong Learner.</t>
+          <t>4.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (38%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0022812</t>
+          <t>CAND_0024466</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>15.9683</v>
+        <v>15.8679</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>4.5 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (79%).  Lifelong Learner.</t>
+          <t>5.2 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0082086</t>
+          <t>CAND_0045027</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>15.9508</v>
+        <v>15.8545</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (85%).</t>
+          <t>3.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0024466</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>15.5263</v>
+        <v>15.7239</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (47%).  Lifelong Learner.</t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0082262</t>
+          <t>CAND_0076251</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>15.0779</v>
+        <v>15.6503</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>5.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (64%).  Lifelong Learner.</t>
+          <t>7.6 yrs exp as Search Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0076251</t>
+          <t>CAND_0082086</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>15.0083</v>
+        <v>15.4026</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>7.6 yrs exp as Search Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (51%).</t>
+          <t>6.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (85%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0091899</t>
+          <t>CAND_0082262</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>14.4385</v>
+        <v>14.8267</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (51%).  Lifelong Learner.</t>
+          <t>5.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (64%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0068892</t>
+          <t>CAND_0091899</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>14.1872</v>
+        <v>14.2946</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (51%).  Lifelong Learner.</t>
+          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0025923</t>
+          <t>CAND_0068892</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>14.0658</v>
+        <v>14.0849</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>5.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (84%).  Lifelong Learner.</t>
+          <t>4.7 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0060257</t>
+          <t>CAND_0025923</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>14.0019</v>
+        <v>13.8265</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%).</t>
+          <t>5.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
@@ -934,443 +934,443 @@
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>13.8787</v>
+        <v>13.7131</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>6.9 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (65%).</t>
+          <t>6.9 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (65%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0010408</t>
+          <t>CAND_0058412</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>13.8609</v>
+        <v>13.3604</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>5.7 yrs exp as Junior ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (36%).  Lifelong Learner.</t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0096104</t>
+          <t>CAND_0062707</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>13.5991</v>
+        <v>13.3478</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>7.0 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (33%).  Lifelong Learner.</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0061156</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>13.5407</v>
+        <v>13.3092</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (43%).</t>
+          <t>6.0 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (39%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0062707</t>
+          <t>CAND_0060257</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>13.2556</v>
+        <v>13.3034</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%).  Lifelong Learner.</t>
+          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0059795</t>
+          <t>CAND_0010408</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>13.2344</v>
+        <v>13.2026</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (75%).  Lifelong Learner.</t>
+          <t>5.7 yrs exp as Junior ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (36%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0088526</t>
+          <t>CAND_0096104</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>13.1835</v>
+        <v>13.0592</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). Fast-track promotions.</t>
+          <t>7.0 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (33%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0061156</t>
+          <t>CAND_0088526</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>13.1417</v>
+        <v>13.0194</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (39%).</t>
+          <t>4.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "\ud83d\udcc8 High Velocity", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0015097</t>
+          <t>CAND_0059795</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>12.8625</v>
+        <v>12.8571</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (69%).</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (75%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0077552</t>
+          <t>CAND_0015097</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>12.6173</v>
+        <v>12.6611</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>3.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%).  Lifelong Learner.</t>
+          <t>6.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0091348</t>
+          <t>CAND_0077552</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>12.563</v>
+        <v>12.5888</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (86%).  Lifelong Learner.</t>
+          <t>3.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0013665</t>
+          <t>CAND_0091348</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>12.2595</v>
+        <v>12.441</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%).  Lifelong Learner.</t>
+          <t>3.7 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (86%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0078810</t>
+          <t>CAND_0074325</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>12.2595</v>
+        <v>12.352</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>6.9 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%).</t>
+          <t>3.9 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0010541</t>
+          <t>CAND_0074648</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>12.229</v>
+        <v>12.2284</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>6.2 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (59%).  Lifelong Learner.</t>
+          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (82%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0005269</t>
+          <t>CAND_0078810</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>12.21</v>
+        <v>12.1993</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%).  Lifelong Learner.</t>
+          <t>6.9 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0043312</t>
+          <t>CAND_0005269</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>12.2076</v>
+        <v>11.9801</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>4.2 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (73%).</t>
+          <t>6.1 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0007008</t>
+          <t>CAND_0010541</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>12.1736</v>
+        <v>11.9405</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (66%).  Lifelong Learner.</t>
+          <t>6.2 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (59%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0046313</t>
+          <t>CAND_0007008</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>12.0981</v>
+        <v>11.9211</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (45%).  Lifelong Learner.</t>
+          <t>3.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (66%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0074325</t>
+          <t>CAND_0046313</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>12.0855</v>
+        <v>11.9209</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (47%).</t>
+          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (45%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0009516</t>
+          <t>CAND_0013665</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>12.0486</v>
+        <v>11.8241</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>6.9 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (34%).  Lifelong Learner.</t>
+          <t>5.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0074648</t>
+          <t>CAND_0009516</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>12.0098</v>
+        <v>11.7054</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (82%).</t>
+          <t>6.9 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (34%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0003609</t>
+          <t>CAND_0079688</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>11.9048</v>
+        <v>11.6653</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (50%).  Lifelong Learner.</t>
+          <t>3.3 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0079688</t>
+          <t>CAND_0089249</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>11.7606</v>
+        <v>11.6498</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3.3 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (69%).  Lifelong Learner.</t>
+          <t>3.1 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0077956</t>
+          <t>CAND_0003609</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>11.6738</v>
+        <v>11.6453</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>6.4 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (88%).  Lifelong Learner.</t>
+          <t>6.1 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (50%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0089249</t>
+          <t>CAND_0043312</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>11.5768</v>
+        <v>11.5914</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>3.1 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (47%).</t>
+          <t>4.2 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
@@ -1384,407 +1384,407 @@
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>11.5596</v>
+        <v>11.3966</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%).</t>
+          <t>6.0 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0018961</t>
+          <t>CAND_0072032</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>11.4328</v>
+        <v>11.3684</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>5.0 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (26%).</t>
+          <t>6.1 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (38%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0072032</t>
+          <t>CAND_0018961</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>11.3558</v>
+        <v>11.34</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (38%).</t>
+          <t>5.0 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (26%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0073007</t>
+          <t>CAND_0088878</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>11.3265</v>
+        <v>11.3235</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%).  Lifelong Learner.</t>
+          <t>4.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (31%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0026942</t>
+          <t>CAND_0077956</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>11.3171</v>
+        <v>11.2998</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%).  Lifelong Learner.</t>
+          <t>6.4 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0082913</t>
+          <t>CAND_0008218</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>11.2736</v>
+        <v>11.174</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>5.5 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%).</t>
+          <t>7.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (39%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0088878</t>
+          <t>CAND_0082913</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>11.2392</v>
+        <v>11.1647</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>4.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (31%).  Lifelong Learner.</t>
+          <t>5.5 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0008218</t>
+          <t>CAND_0073007</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>11.1902</v>
+        <v>11.0339</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>7.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (39%).</t>
+          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0077498</t>
+          <t>CAND_0075502</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>11.0874</v>
+        <v>10.8774</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (89%).  Lifelong Learner.</t>
+          <t>3.3 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0060315</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>11.0303</v>
+        <v>10.7622</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>6.8 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%).</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (63%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0024947</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>11.0223</v>
+        <v>10.7408</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%).</t>
+          <t>6.8 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>11.0203</v>
+        <v>10.7393</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (81%).</t>
+          <t>7.1 yrs exp as Applied ML Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (61%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0075502</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>10.9718</v>
+        <v>10.7376</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>3.3 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%).</t>
+          <t>6.1 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (81%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0002344</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>10.9629</v>
+        <v>10.7239</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%).  Lifelong Learner.</t>
+          <t>4.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0002344</t>
+          <t>CAND_0077498</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>10.9202</v>
+        <v>10.7199</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (83%).</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (89%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0024947</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>10.8376</v>
+        <v>10.6434</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>7.1 yrs exp as Applied ML Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (61%).</t>
+          <t>6.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0079550</t>
+          <t>CAND_0012988</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>10.7789</v>
+        <v>10.5653</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (88%).  Lifelong Learner.</t>
+          <t>4.3 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0060315</t>
+          <t>CAND_0026942</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>10.7168</v>
+        <v>10.4784</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (63%).  Lifelong Learner.</t>
+          <t>6.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0025882</t>
+          <t>CAND_0079550</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>10.6615</v>
+        <v>10.3863</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%).  Lifelong Learner.</t>
+          <t>3.9 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0098952</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>10.6221</v>
+        <v>10.3484</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>5.5 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (66%).  Lifelong Learner.</t>
+          <t>5.0 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0012988</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>10.6132</v>
+        <v>10.3175</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>4.3 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%).</t>
+          <t>5.2 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0025882</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>10.4847</v>
+        <v>10.29</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>5.0 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%).</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0002793</t>
+          <t>CAND_0098952</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>10.3095</v>
+        <v>10.1637</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>5.5 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (77%).</t>
+          <t>5.5 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (66%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
@@ -1798,119 +1798,119 @@
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>10.2182</v>
+        <v>10.0344</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>5.3 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (52%).  Lifelong Learner.</t>
+          <t>5.3 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (52%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0070525</t>
+          <t>CAND_0061175</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>9.8941</v>
+        <v>9.912000000000001</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (93%).  Lifelong Learner.</t>
+          <t>6.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0080315</t>
         </is>
       </c>
       <c r="B79" t="n">
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>9.8934</v>
+        <v>9.788600000000001</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>6.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%).</t>
+          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0065139</t>
+          <t>CAND_0002793</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>9.869199999999999</v>
+        <v>9.77</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (82%).  Lifelong Learner.</t>
+          <t>5.5 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (77%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0064331</t>
+          <t>CAND_0065139</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>9.8558</v>
+        <v>9.7301</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>4.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (74%).</t>
+          <t>5.2 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (82%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0080315</t>
+          <t>CAND_0024630</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>9.793799999999999</v>
+        <v>9.6967</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%).  Lifelong Learner.</t>
+          <t>3.0 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0009200</t>
+          <t>CAND_0064331</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>9.715299999999999</v>
+        <v>9.6548</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>5.7 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (32%).</t>
+          <t>4.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (74%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
@@ -1924,65 +1924,65 @@
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>9.6838</v>
+        <v>9.595499999999999</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>6.2 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (64%).  Lifelong Learner.</t>
+          <t>6.2 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (64%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0014063</t>
+          <t>CAND_0042441</t>
         </is>
       </c>
       <c r="B85" t="n">
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>9.588699999999999</v>
+        <v>9.509600000000001</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (69%).</t>
+          <t>4.1 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0081480</t>
+          <t>CAND_0070525</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>9.5494</v>
+        <v>9.4587</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Computer Vision Engineer. Strong semantic alignment with AI system requirements. Highly responsive (85%).</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (93%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0091890</t>
+          <t>CAND_0077881</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>9.4201</v>
+        <v>9.3499</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (49%).</t>
+          <t>4.6 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
@@ -1996,11 +1996,11 @@
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>9.351100000000001</v>
+        <v>9.314</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (77%).  Lifelong Learner.</t>
+          <t>3.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (77%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
@@ -2014,227 +2014,227 @@
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>9.2898</v>
+        <v>9.3086</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (32%).</t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (32%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0077881</t>
+          <t>CAND_0023076</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>9.2624</v>
+        <v>9.307</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (30%).</t>
+          <t>3.7 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (61%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0056584</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>9.238899999999999</v>
+        <v>9.2597</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (57%).</t>
+          <t>3.5 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0031306</t>
+          <t>CAND_0072721</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>9.235900000000001</v>
+        <v>9.208399999999999</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>3.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%).  Lifelong Learner.</t>
+          <t>3.7 yrs exp as Data Scientist. Strong semantic alignment with AI system requirements. Highly responsive (53%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0091745</t>
+          <t>CAND_0091890</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>9.208600000000001</v>
+        <v>9.1914</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>5.9 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (53%).</t>
+          <t>4.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (49%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0072721</t>
+          <t>CAND_0051486</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>9.2029</v>
+        <v>9.073700000000001</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as Data Scientist. Strong semantic alignment with AI system requirements. Highly responsive (53%).  Lifelong Learner.</t>
+          <t>5.9 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (60%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0056584</t>
+          <t>CAND_0081480</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>9.1015</v>
+        <v>9.0588</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>3.5 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (69%).</t>
+          <t>5.6 yrs exp as Computer Vision Engineer. Strong semantic alignment with AI system requirements. Highly responsive (85%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0008628</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>9.0868</v>
+        <v>9.053599999999999</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>3.2 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%).  Lifelong Learner.</t>
+          <t>5.8 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (57%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0080597</t>
+          <t>CAND_0052498</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>9.085000000000001</v>
+        <v>9.033099999999999</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>4.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (33%).  Lifelong Learner.</t>
+          <t>4.7 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0052498</t>
+          <t>CAND_0008628</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>9.0349</v>
+        <v>9.0318</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (28%).  Lifelong Learner.</t>
+          <t>3.2 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0091229</t>
+          <t>CAND_0031306</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>8.936500000000001</v>
+        <v>9.0054</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>7.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (35%).</t>
+          <t>3.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0059520</t>
+          <t>CAND_0080597</t>
         </is>
       </c>
       <c r="B100" t="n">
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>8.930999999999999</v>
+        <v>8.8993</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>4.3 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (36%).  Lifelong Learner.</t>
+          <t>4.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (33%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0012632</t>
+          <t>CAND_0091745</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>8.8279</v>
+        <v>8.8752</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (53%).  Lifelong Learner.</t>
+          <t>5.9 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (53%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The God-Tier Omni-Architecture: Plotly Radar Charts, Leadership NLP, Temporal Consistency, Geo-Viability
</commit_message>
<xml_diff>
--- a/team_PJ2001_IND.xlsx
+++ b/team_PJ2001_IND.xlsx
@@ -441,486 +441,486 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0044222</t>
+          <t>CAND_0018549</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>26.4706</v>
+        <v>26.6879</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7.7 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (60%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 26687.9}</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0091534</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>25.9109</v>
+        <v>24.6521</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>16.9 yrs exp as AI Engineer. Built the document ingestion pipeline (chunking, embedding via OpenAI embeddings, storing in Pinecon... Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>16.6 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 0.9, "semantic_score": 24652.1}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0062247</t>
+          <t>CAND_0061265</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>23.4074</v>
+        <v>23.3438</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.3 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
+          <t>6.6 yrs exp as Recommendation Systems Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (94%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 23343.8}</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0012957</t>
+          <t>CAND_0011162</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>23.3754</v>
+        <v>23.216</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (67%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (75%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 23216.0}</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0012957</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>21.8629</v>
+        <v>22.665</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.8 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (77%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.9 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (67%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 22665.0}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0011162</t>
+          <t>CAND_0075249</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>21.4646</v>
+        <v>22.2833</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (75%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
+          <t>6.2 yrs exp as Applied ML Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (82%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 22283.3}</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0079284</t>
+          <t>CAND_0062247</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>21.3721</v>
+        <v>22.1829</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as Machine Learning Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
+          <t>7.3 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 22182.9}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0013536</t>
+          <t>CAND_0000031</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>21.1153</v>
+        <v>22.0766</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>14.1 yrs exp as Applied ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (87%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.0 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (91%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 22076.6}</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0099806</t>
+          <t>CAND_0061339</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>21.0775</v>
+        <v>21.98</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (76%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (90%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 21980.0}</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0061339</t>
+          <t>CAND_0022812</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>20.9492</v>
+        <v>21.6657</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>4.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (90%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.5 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21665.7}</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0091534</t>
+          <t>CAND_0053695</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>20.6699</v>
+        <v>21.5953</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>16.6 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (60%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21595.3}</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0030827</t>
+          <t>CAND_0013536</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>20.6129</v>
+        <v>21.4087</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Data Scientist. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (52%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>14.1 yrs exp as Applied ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (87%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21408.7}</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0065195</t>
+          <t>CAND_0015528</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>20.5058</v>
+        <v>21.0425</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>5.1 yrs exp as Search Engineer. Built the document ingestion pipeline (chunking, embedding via OpenAI embeddings, storing in Pinecon... Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
+          <t>7.4 yrs exp as Applied ML Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (53%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21042.5}</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0064904</t>
+          <t>CAND_0049538</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>18.8519</v>
+        <v>20.986</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as AI Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.8 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 20986.0}</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0009024</t>
+          <t>CAND_0030953</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>18.0062</v>
+        <v>20.5424</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (46%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
+          <t>7.8 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (63%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 20542.4}</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0024620</t>
+          <t>CAND_0079284</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>16.3938</v>
+        <v>19.7564</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>5.9 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.9 yrs exp as Machine Learning Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 19756.4}</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0022812</t>
+          <t>CAND_0099806</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>16.0565</v>
+        <v>19.3483</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.5 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.6 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (76%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 19348.3}</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0060886</t>
+          <t>CAND_0064904</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>15.8784</v>
+        <v>18.914</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (38%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.9 yrs exp as AI Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 18914.0}</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0024466</t>
+          <t>CAND_0016163</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>15.8679</v>
+        <v>18.6949</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.7 yrs exp as Applied ML Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 18694.9}</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0045027</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>15.8545</v>
+        <v>16.3449</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>7.1 yrs exp as Applied ML Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (61%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 16344.9}</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0049978</t>
+          <t>CAND_0043228</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>15.7239</v>
+        <v>16.2716</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.8 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 16271.6}</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0076251</t>
+          <t>CAND_0060886</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>15.6503</v>
+        <v>15.4991</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>7.6 yrs exp as Search Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni"}</t>
+          <t>4.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (38%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 15499.1}</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0082086</t>
+          <t>CAND_0070202</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>15.4026</v>
+        <v>15.4623</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (85%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.1 yrs exp as Machine Learning Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (60%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 15462.3}</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0082262</t>
+          <t>CAND_0068892</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>14.8267</v>
+        <v>14.9155</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>5.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (64%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.7 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 14915.5}</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0091899</t>
+          <t>CAND_0082086</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>14.2946</v>
+        <v>14.6684</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (85%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 14668.4}</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0068892</t>
+          <t>CAND_0074325</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>14.0849</v>
+        <v>14.6322</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.9 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 14632.2}</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0025923</t>
+          <t>CAND_0004402</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>13.8265</v>
+        <v>14.2941</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.0 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 14294.1}</t>
         </is>
       </c>
     </row>
@@ -934,173 +934,173 @@
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>13.7131</v>
+        <v>14.0341</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>6.9 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (65%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.9 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (65%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 14034.1}</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0020049</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>13.3604</v>
+        <v>13.9969</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.8 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13996.9}</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CAND_0062707</t>
+          <t>CAND_0059795</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>13.3478</v>
+        <v>13.4401</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (75%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13440.1}</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0061156</t>
+          <t>CAND_0045027</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>13.3092</v>
+        <v>13.3752</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (39%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 13375.2}</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0060257</t>
+          <t>CAND_0043676</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>13.3034</v>
+        <v>13.3249</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.1 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (65%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "\ud83d\udcc8 High Velocity", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 13324.9}</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0010408</t>
+          <t>CAND_0061696</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>13.2026</v>
+        <v>13.1721</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>5.7 yrs exp as Junior ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (36%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.5 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13172.1}</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0096104</t>
+          <t>CAND_0087744</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>13.0592</v>
+        <v>13.1643</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>7.0 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (33%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13164.3}</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0088526</t>
+          <t>CAND_0010408</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>13.0194</v>
+        <v>13.1114</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "\ud83d\udcc8 High Velocity", "elite": "Standard"}</t>
+          <t>5.7 yrs exp as Junior ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (36%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 13111.4}</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0059795</t>
+          <t>CAND_0066791</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>12.8571</v>
+        <v>13.1109</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (75%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (42%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13110.9}</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0015097</t>
+          <t>CAND_0049978</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>12.6611</v>
+        <v>13.0353</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 13035.3}</t>
         </is>
       </c>
     </row>
@@ -1114,335 +1114,335 @@
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>12.5888</v>
+        <v>12.9502</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 12950.2}</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0091348</t>
+          <t>CAND_0020350</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>12.441</v>
+        <v>12.5839</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (86%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.8 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (57%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12583.9}</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0074325</t>
+          <t>CAND_0061156</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>12.352</v>
+        <v>12.5666</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.0 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (39%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12566.6}</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0074648</t>
+          <t>CAND_0082262</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>12.2284</v>
+        <v>12.5445</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (82%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (64%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 12544.5}</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0078810</t>
+          <t>CAND_0091899</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>12.1993</v>
+        <v>12.5396</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>6.9 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12539.6}</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0005269</t>
+          <t>CAND_0062707</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>11.9801</v>
+        <v>12.5139</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12513.9}</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0010541</t>
+          <t>CAND_0024947</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>11.9405</v>
+        <v>12.3851</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>6.2 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (59%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12385.1}</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0007008</t>
+          <t>CAND_0024630</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>11.9211</v>
+        <v>12.3677</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (66%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.0 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 12367.7}</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0046313</t>
+          <t>CAND_0060257</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>11.9209</v>
+        <v>12.3313</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (45%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12331.3}</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0013665</t>
+          <t>CAND_0080315</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>11.8241</v>
+        <v>11.9699</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11969.9}</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0009516</t>
+          <t>CAND_0096104</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>11.7054</v>
+        <v>11.9626</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>6.9 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (34%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>7.0 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (33%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 11962.6}</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0079688</t>
+          <t>CAND_0042441</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>11.6653</v>
+        <v>11.9264</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>3.3 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.1 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 11926.4}</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0089249</t>
+          <t>CAND_0023076</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>11.6498</v>
+        <v>11.8636</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3.1 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.7 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (61%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11863.6}</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0003609</t>
+          <t>CAND_0058412</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>11.6453</v>
+        <v>11.5899</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (50%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11589.9}</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0043312</t>
+          <t>CAND_0073007</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>11.5914</v>
+        <v>11.3341</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>4.2 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11334.1}</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0004402</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>11.3966</v>
+        <v>11.3275</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.2 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11327.5}</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0072032</t>
+          <t>CAND_0003609</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>11.3684</v>
+        <v>11.2284</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (38%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.1 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (50%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11228.4}</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0018961</t>
+          <t>CAND_0078810</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>11.34</v>
+        <v>11.1652</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>5.0 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (26%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.9 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 11165.2}</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0088878</t>
+          <t>CAND_0089249</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>11.3235</v>
+        <v>11.1444</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>4.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (31%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.1 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11144.4}</t>
         </is>
       </c>
     </row>
@@ -1456,515 +1456,515 @@
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>11.2998</v>
+        <v>11.1421</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>6.4 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.4 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 11142.1}</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0008218</t>
+          <t>CAND_0069638</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>11.174</v>
+        <v>11.1111</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>7.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (39%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.2 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (64%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11111.1}</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0082913</t>
+          <t>CAND_0025882</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>11.1647</v>
+        <v>10.9381</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>5.5 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10938.1}</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0073007</t>
+          <t>CAND_0088526</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>11.0339</v>
+        <v>10.793</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "\ud83d\udcc8 High Velocity", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10793.0}</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0075502</t>
+          <t>CAND_0008218</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>10.8774</v>
+        <v>10.7913</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>3.3 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>7.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (39%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10791.3}</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0060315</t>
+          <t>CAND_0074648</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>10.7622</v>
+        <v>10.7554</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (63%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (82%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10755.4}</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0043228</t>
+          <t>CAND_0007008</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>10.7408</v>
+        <v>10.5715</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>6.8 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (66%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10571.5}</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0039383</t>
+          <t>CAND_0091348</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>10.7393</v>
+        <v>10.5683</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>7.1 yrs exp as Applied ML Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (61%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.7 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (86%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10568.3}</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0043860</t>
+          <t>CAND_0009516</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>10.7376</v>
+        <v>10.5664</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (81%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.9 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (34%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10566.4}</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0002344</t>
+          <t>CAND_0013665</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>10.7239</v>
+        <v>10.5315</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10531.5}</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0077498</t>
+          <t>CAND_0088878</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>10.7199</v>
+        <v>10.5039</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (89%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (31%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10503.9}</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0024947</t>
+          <t>CAND_0060315</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>10.6434</v>
+        <v>10.4167</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (63%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10416.7}</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0012988</t>
+          <t>CAND_0002344</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>10.5653</v>
+        <v>10.2695</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>4.3 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10269.5}</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0026942</t>
+          <t>CAND_0072032</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>10.4784</v>
+        <v>10.2666</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.1 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (38%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10266.6}</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0079550</t>
+          <t>CAND_0003841</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>10.3863</v>
+        <v>10.2302</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.0 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10230.2}</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0003841</t>
+          <t>CAND_0010541</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>10.3484</v>
+        <v>10.2002</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>5.0 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.2 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (59%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10200.2}</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0046313</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>10.3175</v>
+        <v>10.1673</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (45%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10167.3}</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0025882</t>
+          <t>CAND_0060835</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>10.29</v>
+        <v>10.1064</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (32%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10106.4}</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0098952</t>
+          <t>CAND_0043860</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>10.1637</v>
+        <v>10.0864</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>5.5 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (66%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.1 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (81%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10086.4}</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0016657</t>
+          <t>CAND_0070525</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>10.0344</v>
+        <v>10.0298</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>5.3 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (52%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (93%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10029.8}</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0061175</t>
+          <t>CAND_0052498</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>9.912000000000001</v>
+        <v>10.016</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>6.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.7 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10016.0}</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0080315</t>
+          <t>CAND_0064331</t>
         </is>
       </c>
       <c r="B79" t="n">
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>9.788600000000001</v>
+        <v>9.953099999999999</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (74%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 9953.1}</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0002793</t>
+          <t>CAND_0043312</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>9.77</v>
+        <v>9.951700000000001</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>5.5 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (77%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.2 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9951.7}</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0065139</t>
+          <t>CAND_0075502</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>9.7301</v>
+        <v>9.951700000000001</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (82%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.3 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9951.7}</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0024630</t>
+          <t>CAND_0015967</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>9.6967</v>
+        <v>9.8428</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>3.0 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (45%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 9842.8}</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0064331</t>
+          <t>CAND_0079688</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>9.6548</v>
+        <v>9.803900000000001</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>4.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (74%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.3 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9803.9}</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0069638</t>
+          <t>CAND_0084161</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>9.595499999999999</v>
+        <v>9.773199999999999</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>6.2 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (64%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (77%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9773.2}</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0042441</t>
+          <t>CAND_0012988</t>
         </is>
       </c>
       <c r="B85" t="n">
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>9.509600000000001</v>
+        <v>9.688599999999999</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>4.1 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.3 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 9688.6}</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0070525</t>
+          <t>CAND_0018961</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>9.4587</v>
+        <v>9.678599999999999</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (93%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.0 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (26%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 9678.6}</t>
         </is>
       </c>
     </row>
@@ -1978,263 +1978,263 @@
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>9.3499</v>
+        <v>9.616</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.6 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9616.0}</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0084161</t>
+          <t>CAND_0032955</t>
         </is>
       </c>
       <c r="B88" t="n">
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>9.314</v>
+        <v>9.3841</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (77%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.2 yrs exp as Computer Vision Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (26%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9384.1}</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0060835</t>
+          <t>CAND_0077498</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>9.3086</v>
+        <v>9.2372</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (32%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (89%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9237.2}</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0023076</t>
+          <t>CAND_0034767</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>9.307</v>
+        <v>9.2126</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (61%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.5 yrs exp as ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9212.6}</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0056584</t>
+          <t>CAND_0079550</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>9.2597</v>
+        <v>9.123799999999999</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>3.5 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.9 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9123.8}</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0072721</t>
+          <t>CAND_0031306</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>9.208399999999999</v>
+        <v>9.1214</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as Data Scientist. Strong semantic alignment with AI system requirements. Highly responsive (53%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9121.4}</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0091890</t>
+          <t>CAND_0052082</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>9.1914</v>
+        <v>9.023400000000001</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (49%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>3.1 yrs exp as Computer Vision Engineer. Strong semantic alignment with AI system requirements. Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9023.4}</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0051486</t>
+          <t>CAND_0091890</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>9.073700000000001</v>
+        <v>8.9497</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>5.9 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (60%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (49%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8949.7}</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0081480</t>
+          <t>CAND_0026942</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>9.0588</v>
+        <v>8.8704</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Computer Vision Engineer. Strong semantic alignment with AI system requirements. Highly responsive (85%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 8870.4}</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0020350</t>
+          <t>CAND_0012888</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>9.053599999999999</v>
+        <v>8.8652</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (57%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.4 yrs exp as Junior ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8865.2}</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0052498</t>
+          <t>CAND_0068081</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>9.033099999999999</v>
+        <v>8.802300000000001</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.2 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (31%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8802.3}</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0008628</t>
+          <t>CAND_0080597</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>9.0318</v>
+        <v>8.7555</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>3.2 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (33%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8755.5}</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0031306</t>
+          <t>CAND_0067041</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>9.0054</v>
+        <v>8.6958</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>3.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.9 yrs exp as Data Scientist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (34%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8695.8}</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0080597</t>
+          <t>CAND_0072410</t>
         </is>
       </c>
       <c r="B100" t="n">
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>8.8993</v>
+        <v>8.6317</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>4.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (33%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>4.9 yrs exp as ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8631.7}</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0091745</t>
+          <t>CAND_0012632</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>8.8752</v>
+        <v>8.5839</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>5.9 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (53%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard"}</t>
+          <t>6.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (53%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8583.9}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The Singularity: Free/Open-Source Personality Synthesizer, GenAI Summaries, Graphviz Knowledge Graph
</commit_message>
<xml_diff>
--- a/team_PJ2001_IND.xlsx
+++ b/team_PJ2001_IND.xlsx
@@ -452,7 +452,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 26687.9}</t>
+          <t>6.8 yrs exp as Recommendation Systems Engineer. Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 26687.9, "personality": {"conscientiousness": 79, "openness": 35, "extraversion": 48, "agreeableness": 61}, "exec_summary": "The candidate is a highly qualified Recommendation Systems Engineer with 6.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 26687.9. Beyond technical skills, they exhibit an exceptionally stable career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (79%) and openness (35%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Computer Vision", "Weaviate", "Kubernetes", "Elasticsearch", "BigQuery"]}</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>16.6 yrs exp as AI Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 0.9, "semantic_score": 24652.1}</t>
+          <t>16.6 yrs exp as AI Engineer. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 0.9, "semantic_score": 24652.1, "personality": {"conscientiousness": 74, "openness": 25, "extraversion": 82, "agreeableness": 92}, "exec_summary": "The candidate is a highly qualified AI Engineer with 16.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 24652.1. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (74%) and openness (25%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Hugging Face Transformers", "scikit-learn", "Diffusion Models", "Qdrant", "Sentence Transformers"]}</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6.6 yrs exp as Recommendation Systems Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (94%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 23343.8}</t>
+          <t>6.6 yrs exp as Recommendation Systems Engineer. Highly responsive (94%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 23343.8, "personality": {"conscientiousness": 93, "openness": 40, "extraversion": 89, "agreeableness": 56}, "exec_summary": "The candidate is a highly qualified Recommendation Systems Engineer with 6.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 23343.8. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (93%) and openness (40%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Qdrant", "SQL", "Accounting", "LangChain", "Learning to Rank"]}</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (75%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 23216.0}</t>
+          <t>5.8 yrs exp as Recommendation Systems Engineer. Highly responsive (75%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 23216.0, "personality": {"conscientiousness": 81, "openness": 92, "extraversion": 67, "agreeableness": 47}, "exec_summary": "The candidate is a highly qualified Recommendation Systems Engineer with 5.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 23216.0. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (81%) and openness (92%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Weights &amp; Biases", "FAISS", "Vector Search", "LangChain", "CNN"]}</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as Search Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (67%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 22665.0}</t>
+          <t>4.9 yrs exp as Search Engineer. Highly responsive (67%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 22665.0, "personality": {"conscientiousness": 80, "openness": 87, "extraversion": 46, "agreeableness": 43}, "exec_summary": "The candidate is a highly qualified Search Engineer with 4.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 22665.0. Beyond technical skills, they exhibit an exceptionally stable career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (80%) and openness (87%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["RAG", "PEFT", "LangChain", "ASR", "Deep Learning"]}</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>6.2 yrs exp as Applied ML Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (82%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 22283.3}</t>
+          <t>6.2 yrs exp as Applied ML Engineer. Highly responsive (82%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 22283.3, "personality": {"conscientiousness": 84, "openness": 35, "extraversion": 68, "agreeableness": 65}, "exec_summary": "The candidate is a highly qualified Applied ML Engineer with 6.2 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 22283.3. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (84%) and openness (35%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Sentence Transformers", "Milvus", "Machine Learning", "Fine-tuning LLMs", "MLflow"]}</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>7.3 yrs exp as AI Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 22182.9}</t>
+          <t>7.3 yrs exp as AI Engineer. Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 22182.9, "personality": {"conscientiousness": 78, "openness": 42, "extraversion": 76, "agreeableness": 89}, "exec_summary": "The candidate is a highly qualified AI Engineer with 7.3 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 22182.9. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (78%) and openness (42%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Image Classification", "OpenCV", "Reinforcement Learning", "ASR", "Pinecone"]}</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (91%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 22076.6}</t>
+          <t>6.0 yrs exp as Recommendation Systems Engineer. Highly responsive (91%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 22076.6, "personality": {"conscientiousness": 85, "openness": 42, "extraversion": 66, "agreeableness": 70}, "exec_summary": "The candidate is a highly qualified Recommendation Systems Engineer with 6.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 22076.6. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (85%) and openness (42%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Go", "MLflow", "FAISS", "Pinecone", "Angular"]}</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4.2 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (90%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 21980.0}</t>
+          <t>4.2 yrs exp as Search Engineer. Highly responsive (90%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 21980.0, "personality": {"conscientiousness": 79, "openness": 35, "extraversion": 92, "agreeableness": 55}, "exec_summary": "The candidate is a highly qualified Search Engineer with 4.2 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 21980.0. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (79%) and openness (35%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Information Retrieval", "YOLO", "Data Pipelines", "Milvus", "BentoML"]}</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>4.5 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21665.7}</t>
+          <t>4.5 yrs exp as Applied ML Engineer. Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21665.7, "personality": {"conscientiousness": 75, "openness": 97, "extraversion": 49, "agreeableness": 64}, "exec_summary": "The candidate is a highly qualified Applied ML Engineer with 4.5 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 21665.7. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (75%) and openness (97%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Weaviate", "Pinecone", "LoRA", "Prompt Engineering", "Qdrant"]}</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Recommendation Systems Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (60%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21595.3}</t>
+          <t>5.8 yrs exp as Recommendation Systems Engineer. Highly responsive (60%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21595.3, "personality": {"conscientiousness": 64, "openness": 37, "extraversion": 83, "agreeableness": 80}, "exec_summary": "The candidate is a highly qualified Recommendation Systems Engineer with 5.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 21595.3. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (64%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["MLOps", "Apache Flink", "GCP", "Pinecone", "CNN"]}</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>14.1 yrs exp as Applied ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (87%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21408.7}</t>
+          <t>14.1 yrs exp as Applied ML Engineer. Highly responsive (87%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21408.7, "personality": {"conscientiousness": 74, "openness": 45, "extraversion": 45, "agreeableness": 53}, "exec_summary": "The candidate is a highly qualified Applied ML Engineer with 14.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 21408.7. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (74%) and openness (45%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["PyTorch", "Prompt Engineering", "LLMs", "NLP", "Embeddings"]}</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>7.4 yrs exp as Applied ML Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (53%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21042.5}</t>
+          <t>7.4 yrs exp as Applied ML Engineer. Highly responsive (53%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 21042.5, "personality": {"conscientiousness": 69, "openness": 92, "extraversion": 75, "agreeableness": 76}, "exec_summary": "The candidate is a highly qualified Applied ML Engineer with 7.4 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 21042.5. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (69%) and openness (92%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Docker", "Weaviate", "BentoML", "Weights &amp; Biases", "LangChain"]}</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 20986.0}</t>
+          <t>5.8 yrs exp as Applied ML Engineer. Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 20986.0, "personality": {"conscientiousness": 69, "openness": 42, "extraversion": 95, "agreeableness": 86}, "exec_summary": "The candidate is a highly qualified Applied ML Engineer with 5.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 20986.0. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (69%) and openness (42%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["LlamaIndex", "Feature Engineering", "MLflow", "Computer Vision", "TTS"]}</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>7.8 yrs exp as Search Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (63%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 20542.4}</t>
+          <t>7.8 yrs exp as Search Engineer. Highly responsive (63%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 20542.4, "personality": {"conscientiousness": 77, "openness": 85, "extraversion": 60, "agreeableness": 56}, "exec_summary": "The candidate is a highly qualified Search Engineer with 7.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 20542.4. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (77%) and openness (85%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["TTS", "MLOps", "Learning to Rank", "Databricks", "Time Series"]}</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as Machine Learning Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 19756.4}</t>
+          <t>4.9 yrs exp as Machine Learning Engineer. Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 19756.4, "personality": {"conscientiousness": 82, "openness": 87, "extraversion": 19, "agreeableness": 89}, "exec_summary": "The candidate is a highly qualified Machine Learning Engineer with 4.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 19756.4. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (82%) and openness (87%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Recommendation Systems", "scikit-learn", "QLoRA", "LlamaIndex", "Illustrator"]}</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (76%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 19348.3}</t>
+          <t>4.6 yrs exp as AI Engineer. Highly responsive (76%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 19348.3, "personality": {"conscientiousness": 83, "openness": 45, "extraversion": 63, "agreeableness": 88}, "exec_summary": "The candidate is a highly qualified AI Engineer with 4.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 19348.3. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (83%) and openness (45%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["LoRA", "OpenCV", "Statistical Modeling", "RAG", "Agile"]}</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as AI Engineer. Built a content recommendation system serving 10M+ users that combined collaborative filtering with ... Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 18914.0}</t>
+          <t>4.9 yrs exp as AI Engineer. Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 18914.0, "personality": {"conscientiousness": 82, "openness": 40, "extraversion": 79, "agreeableness": 49}, "exec_summary": "The candidate is a highly qualified AI Engineer with 4.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 18914.0. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (82%) and openness (40%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Embeddings", "Hugging Face Transformers", "Elasticsearch", "Diffusion Models", "Forecasting"]}</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>6.7 yrs exp as Applied ML Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 18694.9}</t>
+          <t>6.7 yrs exp as Applied ML Engineer. Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "\u2b50 Elite Alumni", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 18694.9, "personality": {"conscientiousness": 87, "openness": 42, "extraversion": 97, "agreeableness": 46}, "exec_summary": "The candidate is a highly qualified Applied ML Engineer with 6.7 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 18694.9. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (87%) and openness (42%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Hugging Face Transformers", "Computer Vision", "gRPC", "Time Series", "Weaviate"]}</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>7.1 yrs exp as Applied ML Engineer. Developed a semantic search feature for an internal knowledge base of ~500K documents... Highly responsive (61%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 16344.9}</t>
+          <t>7.1 yrs exp as Applied ML Engineer. Highly responsive (61%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 16344.9, "personality": {"conscientiousness": 83, "openness": 40, "extraversion": 93, "agreeableness": 40}, "exec_summary": "The candidate is a highly qualified Applied ML Engineer with 7.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 16344.9. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (83%) and openness (40%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["GANs", "FAISS", "ASR", "Kubeflow", "Recommendation Systems"]}</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>6.8 yrs exp as Applied ML Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (41%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 16271.6}</t>
+          <t>6.8 yrs exp as Applied ML Engineer. Highly responsive (41%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 16271.6, "personality": {"conscientiousness": 76, "openness": 45, "extraversion": 73, "agreeableness": 70}, "exec_summary": "The candidate is a highly qualified Applied ML Engineer with 6.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 16271.6. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (76%) and openness (45%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["BigQuery", "NLP", "ASR", "Hugging Face Transformers", "FastAPI"]}</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (38%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 15499.1}</t>
+          <t>4.6 yrs exp as Senior Software Engineer (ML). Highly responsive (38%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 15499.1, "personality": {"conscientiousness": 71, "openness": 85, "extraversion": 41, "agreeableness": 44}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 4.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 15499.1. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (71%) and openness (85%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["FAISS", "Python", "MLflow", "Statistical Modeling", "GANs"]}</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>5.1 yrs exp as Machine Learning Engineer. Owned the ranking layer for an e-commerce search product, evolving it from a hand-tuned scoring func... Highly responsive (60%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 15462.3}</t>
+          <t>5.1 yrs exp as Machine Learning Engineer. Highly responsive (60%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 15462.3, "personality": {"conscientiousness": 71, "openness": 37, "extraversion": 19, "agreeableness": 40}, "exec_summary": "The candidate is a highly qualified Machine Learning Engineer with 5.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 15462.3. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (71%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Microservices", "Object Detection", "OpenCV", "Embeddings", "Qdrant"]}</t>
         </is>
       </c>
     </row>
@@ -866,7 +866,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 14915.5}</t>
+          <t>4.7 yrs exp as Senior Software Engineer (ML). Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 14915.5, "personality": {"conscientiousness": 70, "openness": 87, "extraversion": 87, "agreeableness": 35}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 4.7 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 14915.5. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (70%) and openness (87%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["ETL", "LlamaIndex", "Weaviate", "Pinecone", "Computer Vision"]}</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (85%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 14668.4}</t>
+          <t>6.0 yrs exp as Senior Software Engineer (ML). Highly responsive (85%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 14668.4, "personality": {"conscientiousness": 83, "openness": 35, "extraversion": 91, "agreeableness": 67}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 6.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 14668.4. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (83%) and openness (35%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Feature Engineering", "FAISS", "Speech Recognition", "Pinecone", "Kubeflow"]}</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 14632.2}</t>
+          <t>3.9 yrs exp as AI Research Engineer. Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 14632.2, "personality": {"conscientiousness": 66, "openness": 37, "extraversion": 19, "agreeableness": 48}, "exec_summary": "The candidate is a highly qualified AI Research Engineer with 3.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 14632.2. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (66%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["NLP", "Milvus", "BentoML", "OpenSearch", "Deep Learning"]}</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 14294.1}</t>
+          <t>6.0 yrs exp as AI Research Engineer. Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 14294.1, "personality": {"conscientiousness": 92, "openness": 40, "extraversion": 49, "agreeableness": 66}, "exec_summary": "The candidate is a highly qualified AI Research Engineer with 6.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 14294.1. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (92%) and openness (40%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["TypeScript", "TTS", "OpenSearch", "Speech Recognition", "Object Detection"]}</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>6.9 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (65%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 14034.1}</t>
+          <t>6.9 yrs exp as Senior Software Engineer (ML). Highly responsive (65%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 14034.1, "personality": {"conscientiousness": 72, "openness": 37, "extraversion": 88, "agreeableness": 42}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 6.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 14034.1. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (72%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Machine Learning", "GraphQL", "Webpack", "CSS", "Kubeflow"]}</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3.8 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13996.9}</t>
+          <t>3.8 yrs exp as Senior Software Engineer (ML). Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13996.9, "personality": {"conscientiousness": 72, "openness": 92, "extraversion": 35, "agreeableness": 49}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 3.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 13996.9. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (72%) and openness (92%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Data Pipelines", "Reinforcement Learning", "Feature Engineering", "Information Retrieval", "OpenSearch"]}</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (75%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13440.1}</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Highly responsive (75%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13440.1, "personality": {"conscientiousness": 70, "openness": 85, "extraversion": 78, "agreeableness": 62}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 13440.1. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (70%) and openness (85%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["LangChain", "JavaScript", "LLMs", "GANs", "Speech Recognition"]}</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3.0 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 13375.2}</t>
+          <t>3.0 yrs exp as Senior Software Engineer (ML). Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 13375.2, "personality": {"conscientiousness": 78, "openness": 92, "extraversion": 43, "agreeableness": 65}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 3.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 13375.2. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (78%) and openness (92%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Milvus", "Terraform", "Image Classification", "MLflow", "Sentence Transformers"]}</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (65%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "\ud83d\udcc8 High Velocity", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 13324.9}</t>
+          <t>6.1 yrs exp as Senior Software Engineer (ML). Highly responsive (65%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "\ud83d\udcc8 High Velocity", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 13324.9, "personality": {"conscientiousness": 80, "openness": 90, "extraversion": 92, "agreeableness": 82}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 6.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 13324.9. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (80%) and openness (90%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire. Fast-track promotions detected. They are highly responsive and ready to interview.", "skills": ["ASR", "QLoRA", "scikit-learn", "PEFT", "Diffusion Models"]}</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3.5 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13172.1}</t>
+          <t>3.5 yrs exp as Senior Software Engineer (ML). Highly responsive (78%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13172.1, "personality": {"conscientiousness": 81, "openness": 30, "extraversion": 48, "agreeableness": 89}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 3.5 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 13172.1. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (81%) and openness (30%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Speech Recognition", "Microservices", "pgvector", "Embeddings", "Weaviate"]}</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13164.3}</t>
+          <t>3.9 yrs exp as Senior Software Engineer (ML). Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13164.3, "personality": {"conscientiousness": 87, "openness": 37, "extraversion": 34, "agreeableness": 94}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 3.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 13164.3. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (87%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Speech Recognition", "Accounting", "LangChain", "Pinecone", "PyTorch"]}</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>5.7 yrs exp as Junior ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (36%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 13111.4}</t>
+          <t>5.7 yrs exp as Junior ML Engineer. Highly responsive (36%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 13111.4, "personality": {"conscientiousness": 74, "openness": 85, "extraversion": 87, "agreeableness": 43}, "exec_summary": "The candidate is a highly qualified Junior ML Engineer with 5.7 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 13111.4. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (74%) and openness (85%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Kubeflow", "TTS", "Deep Learning", "Hugging Face Transformers", "Azure"]}</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (42%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13110.9}</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Highly responsive (42%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 13110.9, "personality": {"conscientiousness": 59, "openness": 45, "extraversion": 27, "agreeableness": 31}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 13110.9. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (59%) and openness (45%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["BM25", "FastAPI", "Django", "BigQuery", "Python"]}</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 13035.3}</t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Highly responsive (71%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 13035.3, "personality": {"conscientiousness": 88, "openness": 40, "extraversion": 54, "agreeableness": 60}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 6.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 13035.3. Beyond technical skills, they exhibit an exceptionally stable career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (88%) and openness (40%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Deep Learning", "Weaviate", "BM25", "GANs", "LoRA"]}</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (54%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 12950.2}</t>
+          <t>3.4 yrs exp as Senior Software Engineer (ML). Highly responsive (54%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 12950.2, "personality": {"conscientiousness": 68, "openness": 82, "extraversion": 49, "agreeableness": 77}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 3.4 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 12950.2. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (68%) and openness (82%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["MLOps", "TTS", "Statistical Modeling", "GANs", "Next.js"]}</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as AI Engineer. Strong semantic alignment with AI system requirements. Highly responsive (57%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12583.9}</t>
+          <t>5.8 yrs exp as AI Engineer. Highly responsive (57%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12583.9, "personality": {"conscientiousness": 84, "openness": 37, "extraversion": 49, "agreeableness": 79}, "exec_summary": "The candidate is a highly qualified AI Engineer with 5.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 12583.9. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (84%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Content Writing", "MLOps", "NLP", "GANs", "LoRA"]}</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (39%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12566.6}</t>
+          <t>6.0 yrs exp as Senior Software Engineer (ML). Highly responsive (39%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12566.6, "personality": {"conscientiousness": 77, "openness": 35, "extraversion": 49, "agreeableness": 29}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 6.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 12566.6. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (77%) and openness (35%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Airflow", "OpenSearch", "Weaviate", "pgvector", "LangChain"]}</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>5.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (64%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 12544.5}</t>
+          <t>5.9 yrs exp as Senior Software Engineer (ML). Highly responsive (64%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 12544.5, "personality": {"conscientiousness": 80, "openness": 77, "extraversion": 9, "agreeableness": 82}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 12544.5. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (80%) and openness (77%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["LangChain", "Python", "TTS", "QLoRA", "CNN"]}</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12539.6}</t>
+          <t>5.8 yrs exp as Senior Software Engineer (ML). Highly responsive (51%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12539.6, "personality": {"conscientiousness": 77, "openness": 82, "extraversion": 49, "agreeableness": 50}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 12539.6. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (77%) and openness (82%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Statistical Modeling", "Semantic Search", "Apache Flink", "Computer Vision", "Sentence Transformers"]}</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12513.9}</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12513.9, "personality": {"conscientiousness": 63, "openness": 87, "extraversion": 32, "agreeableness": 40}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 12513.9. Beyond technical skills, they exhibit an exceptionally stable career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (63%) and openness (87%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Elasticsearch", "YOLO", "Speech Recognition", "Python", "Content Writing"]}</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12385.1}</t>
+          <t>6.1 yrs exp as AI Research Engineer. Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12385.1, "personality": {"conscientiousness": 76, "openness": 42, "extraversion": 71, "agreeableness": 89}, "exec_summary": "The candidate is a highly qualified AI Research Engineer with 6.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 12385.1. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (76%) and openness (42%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["YOLO", "Milvus", "Hugging Face Transformers", "Information Retrieval", "Kubeflow"]}</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>3.0 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 12367.7}</t>
+          <t>3.0 yrs exp as AI Research Engineer. Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 12367.7, "personality": {"conscientiousness": 65, "openness": 35, "extraversion": 19, "agreeableness": 31}, "exec_summary": "The candidate is a highly qualified AI Research Engineer with 3.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 12367.7. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (65%) and openness (35%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["TTS", "Computer Vision", "Spark", "BM25", "LangChain"]}</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (56%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12331.3}</t>
+          <t>5.8 yrs exp as AI Specialist. Highly responsive (56%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 12331.3, "personality": {"conscientiousness": 70, "openness": 40, "extraversion": 74, "agreeableness": 53}, "exec_summary": "The candidate is a highly qualified AI Specialist with 5.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 12331.3. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (70%) and openness (40%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Recommendation Systems", "Diffusion Models", "BigQuery", "Terraform", "Vector Search"]}</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1280,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11969.9}</t>
+          <t>4.1 yrs exp as AI Research Engineer. Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11969.9, "personality": {"conscientiousness": 59, "openness": 85, "extraversion": 49, "agreeableness": 64}, "exec_summary": "The candidate is a highly qualified AI Research Engineer with 4.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11969.9. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (59%) and openness (85%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["LangChain", "Object Detection", "Python", "Prompt Engineering", "FastAPI"]}</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>7.0 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (33%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 11962.6}</t>
+          <t>7.0 yrs exp as AI Specialist. Highly responsive (33%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 11962.6, "personality": {"conscientiousness": 68, "openness": 77, "extraversion": 85, "agreeableness": 66}, "exec_summary": "The candidate is a highly qualified AI Specialist with 7.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11962.6. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (68%) and openness (77%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["BM25", "TTS", "Hugging Face Transformers", "MLOps", "CI/CD"]}</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>4.1 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 11926.4}</t>
+          <t>4.1 yrs exp as AI Research Engineer. Highly responsive (72%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 11926.4, "personality": {"conscientiousness": 65, "openness": 85, "extraversion": 19, "agreeableness": 46}, "exec_summary": "The candidate is a highly qualified AI Research Engineer with 4.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11926.4. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (65%) and openness (85%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Illustrator", "Feature Engineering", "Sentence Transformers", "Reinforcement Learning", "RAG"]}</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as AI Research Engineer. Strong semantic alignment with AI system requirements. Highly responsive (61%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11863.6}</t>
+          <t>3.7 yrs exp as AI Research Engineer. Highly responsive (61%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11863.6, "personality": {"conscientiousness": 63, "openness": 40, "extraversion": 19, "agreeableness": 40}, "exec_summary": "The candidate is a highly qualified AI Research Engineer with 3.7 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11863.6. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (63%) and openness (40%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Learning to Rank", "Node.js", "Weights &amp; Biases", "TypeScript", "OpenCV"]}</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11589.9}</t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11589.9, "personality": {"conscientiousness": 70, "openness": 42, "extraversion": 65, "agreeableness": 46}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 6.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11589.9. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (70%) and openness (42%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Embeddings", "Speech Recognition", "Data Science", "Object Detection", "Milvus"]}</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11334.1}</t>
+          <t>5.8 yrs exp as AI Specialist. Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11334.1, "personality": {"conscientiousness": 82, "openness": 85, "extraversion": 83, "agreeableness": 66}, "exec_summary": "The candidate is a highly qualified AI Specialist with 5.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11334.1. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (82%) and openness (85%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Milvus", "BentoML", "PyTorch", "Embeddings", "Computer Vision"]}</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (48%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11327.5}</t>
+          <t>5.2 yrs exp as ML Engineer. Highly responsive (48%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11327.5, "personality": {"conscientiousness": 66, "openness": 82, "extraversion": 85, "agreeableness": 74}, "exec_summary": "The candidate is a highly qualified ML Engineer with 5.2 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11327.5. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (66%) and openness (82%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Haystack", "Image Classification", "Reinforcement Learning", "MongoDB", "Pinecone"]}</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (50%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11228.4}</t>
+          <t>6.1 yrs exp as Senior Software Engineer (ML). Highly responsive (50%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11228.4, "personality": {"conscientiousness": 72, "openness": 85, "extraversion": 82, "agreeableness": 50}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 6.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11228.4. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (72%) and openness (85%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Fine-tuning LLMs", "Object Detection", "Kubeflow", "TTS", "Terraform"]}</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>6.9 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 11165.2}</t>
+          <t>6.9 yrs exp as Senior Software Engineer (ML). Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 11165.2, "personality": {"conscientiousness": 83, "openness": 35, "extraversion": 55, "agreeableness": 50}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 6.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11165.2. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (83%) and openness (35%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Recommendation Systems", "Sentence Transformers", "dbt", "BentoML", "Diffusion Models"]}</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>3.1 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11144.4}</t>
+          <t>3.1 yrs exp as Senior Software Engineer (ML). Highly responsive (47%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11144.4, "personality": {"conscientiousness": 74, "openness": 25, "extraversion": 19, "agreeableness": 33}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 3.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11144.4. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (74%) and openness (25%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["LlamaIndex", "Data Pipelines", "Pinecone", "LangChain", "Time Series"]}</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>6.4 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 11142.1}</t>
+          <t>6.4 yrs exp as Computer Vision Engineer. Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 11142.1, "personality": {"conscientiousness": 93, "openness": 95, "extraversion": 70, "agreeableness": 54}, "exec_summary": "The candidate is a highly qualified Computer Vision Engineer with 6.4 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11142.1. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (93%) and openness (95%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Milvus", "TTS", "SQL", "Weights &amp; Biases", "Hugging Face Transformers"]}</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>6.2 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (64%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11111.1}</t>
+          <t>6.2 yrs exp as Computer Vision Engineer. Highly responsive (64%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 11111.1, "personality": {"conscientiousness": 71, "openness": 77, "extraversion": 61, "agreeableness": 82}, "exec_summary": "The candidate is a highly qualified Computer Vision Engineer with 6.2 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 11111.1. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (71%) and openness (77%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Time Series", "Hadoop", "Semantic Search", "Prompt Engineering", "Feature Engineering"]}</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>5.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10938.1}</t>
+          <t>5.6 yrs exp as Senior Software Engineer (ML). Highly responsive (79%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10938.1, "personality": {"conscientiousness": 82, "openness": 80, "extraversion": 67, "agreeableness": 64}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10938.1. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (82%) and openness (80%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["MLflow", "scikit-learn", "Kubeflow", "FAISS", "Feature Engineering"]}</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "\ud83d\udcc8 High Velocity", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10793.0}</t>
+          <t>4.6 yrs exp as Senior Software Engineer (ML). Highly responsive (80%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "\ud83d\udcc8 High Velocity", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10793.0, "personality": {"conscientiousness": 78, "openness": 37, "extraversion": 87, "agreeableness": 50}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 4.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10793.0. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (78%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire. Fast-track promotions detected. They are highly responsive and ready to interview.", "skills": ["Reinforcement Learning", "Node.js", "LangChain", "MLOps", "CSS"]}</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>7.0 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (39%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10791.3}</t>
+          <t>7.0 yrs exp as Senior Software Engineer (ML). Highly responsive (39%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10791.3, "personality": {"conscientiousness": 61, "openness": 27, "extraversion": 49, "agreeableness": 44}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 7.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10791.3. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (61%) and openness (27%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["TensorFlow", "Forecasting", "SQL", "OpenCV", "Statistical Modeling"]}</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>4.1 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (82%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10755.4}</t>
+          <t>4.1 yrs exp as AI Research Engineer. Highly responsive (82%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10755.4, "personality": {"conscientiousness": 76, "openness": 40, "extraversion": 19, "agreeableness": 51}, "exec_summary": "The candidate is a highly qualified AI Research Engineer with 4.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10755.4. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (76%) and openness (40%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["PyTorch", "Weights &amp; Biases", "Data Science", "LangChain", "Forecasting"]}</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (66%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10571.5}</t>
+          <t>3.7 yrs exp as Senior Software Engineer (ML). Highly responsive (66%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10571.5, "personality": {"conscientiousness": 80, "openness": 87, "extraversion": 43, "agreeableness": 58}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 3.7 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10571.5. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (80%) and openness (87%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["LlamaIndex", "Learning to Rank", "BentoML", "GANs", "TensorFlow"]}</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>3.7 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (86%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10568.3}</t>
+          <t>3.7 yrs exp as Senior Software Engineer (ML). Highly responsive (86%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10568.3, "personality": {"conscientiousness": 76, "openness": 87, "extraversion": 19, "agreeableness": 68}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 3.7 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10568.3. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (76%) and openness (87%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["MLflow", "Feature Engineering", "Time Series", "Qdrant", "YOLO"]}</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>6.9 yrs exp as AI Specialist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (34%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10566.4}</t>
+          <t>6.9 yrs exp as AI Specialist. Highly responsive (34%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10566.4, "personality": {"conscientiousness": 62, "openness": 75, "extraversion": 87, "agreeableness": 67}, "exec_summary": "The candidate is a highly qualified AI Specialist with 6.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10566.4. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (62%) and openness (75%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Pinecone", "BentoML", "AWS", "LangChain", "Object Detection"]}</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10531.5}</t>
+          <t>5.2 yrs exp as Senior Software Engineer (ML). Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10531.5, "personality": {"conscientiousness": 87, "openness": 80, "extraversion": 29, "agreeableness": 86}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.2 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10531.5. Beyond technical skills, they exhibit an exceptionally stable career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (87%) and openness (80%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Image Classification", "FastAPI", "Learning to Rank", "ASR", "Terraform"]}</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>4.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (31%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10503.9}</t>
+          <t>4.4 yrs exp as Senior Software Engineer (ML). Highly responsive (31%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10503.9, "personality": {"conscientiousness": 67, "openness": 80, "extraversion": 59, "agreeableness": 25}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 4.4 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10503.9. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (67%) and openness (80%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Statistical Modeling", "MLOps", "Embeddings", "TensorFlow", "Hugging Face Transformers"]}</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1658,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (63%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10416.7}</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Highly responsive (63%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10416.7, "personality": {"conscientiousness": 74, "openness": 95, "extraversion": 49, "agreeableness": 41}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.4 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10416.7. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (74%) and openness (95%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Computer Vision", "Milvus", "Reinforcement Learning", "Hugging Face Transformers", "Fine-tuning LLMs"]}</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10269.5}</t>
+          <t>4.7 yrs exp as Senior Software Engineer (ML). Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10269.5, "personality": {"conscientiousness": 90, "openness": 45, "extraversion": 60, "agreeableness": 51}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 4.7 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10269.5. Beyond technical skills, they exhibit an exceptionally stable career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (90%) and openness (45%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["NLP", "TensorFlow", "Django", "Pinecone", "MLOps"]}</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (38%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10266.6}</t>
+          <t>6.1 yrs exp as AI Specialist. Highly responsive (38%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10266.6, "personality": {"conscientiousness": 75, "openness": 37, "extraversion": 55, "agreeableness": 44}, "exec_summary": "The candidate is a highly qualified AI Specialist with 6.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10266.6. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (75%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Pinecone", "Object Detection", "Java", "Milvus", "Statistical Modeling"]}</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>5.0 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (71%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10230.2}</t>
+          <t>5.0 yrs exp as ML Engineer. Highly responsive (71%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10230.2, "personality": {"conscientiousness": 67, "openness": 40, "extraversion": 63, "agreeableness": 85}, "exec_summary": "The candidate is a highly qualified ML Engineer with 5.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10230.2. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (67%) and openness (40%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Airflow", "Spring Boot", "Diffusion Models", "Statistical Modeling", "Pinecone"]}</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>6.2 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (59%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10200.2}</t>
+          <t>6.2 yrs exp as AI Research Engineer. Highly responsive (59%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10200.2, "personality": {"conscientiousness": 78, "openness": 90, "extraversion": 29, "agreeableness": 54}, "exec_summary": "The candidate is a highly qualified AI Research Engineer with 6.2 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10200.2. Beyond technical skills, they exhibit an exceptionally stable career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (78%) and openness (90%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Pinecone", "GANs", "Weaviate", "Computer Vision", "TTS"]}</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>5.8 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (45%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10167.3}</t>
+          <t>5.8 yrs exp as Senior Software Engineer (ML). Highly responsive (45%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 10167.3, "personality": {"conscientiousness": 73, "openness": 87, "extraversion": 68, "agreeableness": 47}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.8 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10167.3. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (73%) and openness (87%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["YOLO", "Fine-tuning LLMs", "CNN", "LangChain", "pgvector"]}</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>6.6 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (32%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10106.4}</t>
+          <t>6.6 yrs exp as Senior Software Engineer (ML). Highly responsive (32%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10106.4, "personality": {"conscientiousness": 65, "openness": 37, "extraversion": 90, "agreeableness": 26}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 6.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10106.4. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (65%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["SQL", "Flask", "Reinforcement Learning", "PyTorch", "Forecasting"]}</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>6.1 yrs exp as Junior ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (81%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10086.4}</t>
+          <t>6.1 yrs exp as Junior ML Engineer. Highly responsive (81%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10086.4, "personality": {"conscientiousness": 91, "openness": 35, "extraversion": 49, "agreeableness": 90}, "exec_summary": "The candidate is a highly qualified Junior ML Engineer with 6.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10086.4. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (91%) and openness (35%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["pgvector", "Feature Engineering", "Object Detection", "Semantic Search", "Information Retrieval"]}</t>
         </is>
       </c>
     </row>
@@ -1802,7 +1802,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (93%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10029.8}</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Highly responsive (93%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10029.8, "personality": {"conscientiousness": 96, "openness": 80, "extraversion": 59, "agreeableness": 71}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.4 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10029.8. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (96%) and openness (80%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Apache Beam", "Recommendation Systems", "Feature Engineering", "Python", "GANs"]}</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as ML Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10016.0}</t>
+          <t>4.7 yrs exp as ML Engineer. Highly responsive (28%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 10016.0, "personality": {"conscientiousness": 68, "openness": 90, "extraversion": 68, "agreeableness": 39}, "exec_summary": "The candidate is a highly qualified ML Engineer with 4.7 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 10016.0. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (68%) and openness (90%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["PyTorch", "Python", "OpenCV", "QLoRA", "Data Science"]}</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1838,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>4.2 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (74%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 9953.1}</t>
+          <t>4.2 yrs exp as Senior Software Engineer (ML). Highly responsive (74%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 9953.1, "personality": {"conscientiousness": 73, "openness": 37, "extraversion": 49, "agreeableness": 87}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 4.2 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9953.1. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (73%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["LLMs", "BentoML", "Forecasting", "Data Science", "TensorFlow"]}</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>4.2 yrs exp as AI Research Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9951.7}</t>
+          <t>4.2 yrs exp as AI Research Engineer. Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9951.7, "personality": {"conscientiousness": 80, "openness": 42, "extraversion": 56, "agreeableness": 86}, "exec_summary": "The candidate is a highly qualified AI Research Engineer with 4.2 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9951.7. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (80%) and openness (42%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Qdrant", "Image Classification", "Weights &amp; Biases", "Data Science", "Feature Engineering"]}</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>3.3 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9951.7}</t>
+          <t>3.3 yrs exp as Senior Software Engineer (ML). Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9951.7, "personality": {"conscientiousness": 62, "openness": 45, "extraversion": 53, "agreeableness": 40}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 3.3 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9951.7. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (62%) and openness (45%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Qdrant", "Redis", "Computer Vision", "pgvector", "Semantic Search"]}</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (45%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 9842.8}</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Highly responsive (45%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 9842.8, "personality": {"conscientiousness": 59, "openness": 92, "extraversion": 63, "agreeableness": 72}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.4 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9842.8. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (59%) and openness (92%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["QLoRA", "YOLO", "Pinecone", "Object Detection", "Semantic Search"]}</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>3.3 yrs exp as Senior Software Engineer (ML). Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9803.9}</t>
+          <t>3.3 yrs exp as Senior Software Engineer (ML). Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9803.9, "personality": {"conscientiousness": 80, "openness": 95, "extraversion": 45, "agreeableness": 44}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 3.3 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9803.9. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (80%) and openness (95%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Deep Learning", "CNN", "Qdrant", "Haystack", "Sentence Transformers"]}</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1928,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (77%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9773.2}</t>
+          <t>3.9 yrs exp as Senior Software Engineer (ML). Highly responsive (77%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9773.2, "personality": {"conscientiousness": 68, "openness": 80, "extraversion": 9, "agreeableness": 63}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 3.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9773.2. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (68%) and openness (80%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["TTS", "MongoDB", "OpenSearch", "Sentence Transformers", "Python"]}</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>4.3 yrs exp as Senior Software Engineer (ML). Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 9688.6}</t>
+          <t>4.3 yrs exp as Senior Software Engineer (ML). Highly responsive (73%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 0.8, "modesty_score": 1.0, "semantic_score": 9688.6, "personality": {"conscientiousness": 63, "openness": 32, "extraversion": 41, "agreeableness": 61}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 4.3 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9688.6. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (63%) and openness (32%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Feature Engineering", "Hugging Face Transformers", "Forecasting", "Speech Recognition", "PyTorch"]}</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>5.0 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (26%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 9678.6}</t>
+          <t>5.0 yrs exp as AI Specialist. Highly responsive (26%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 9678.6, "personality": {"conscientiousness": 58, "openness": 37, "extraversion": 51, "agreeableness": 38}, "exec_summary": "The candidate is a highly qualified AI Specialist with 5.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9678.6. Beyond technical skills, they exhibit an exceptionally stable career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (58%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Flask", "Reinforcement Learning", "NLP", "Learning to Rank", "Information Retrieval"]}</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>4.6 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9616.0}</t>
+          <t>4.6 yrs exp as Junior ML Engineer. Highly responsive (30%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9616.0, "personality": {"conscientiousness": 66, "openness": 42, "extraversion": 19, "agreeableness": 65}, "exec_summary": "The candidate is a highly qualified Junior ML Engineer with 4.6 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9616.0. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (66%) and openness (42%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Learning to Rank", "Weaviate", "Milvus", "Speech Recognition", "Airflow"]}</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>5.2 yrs exp as Computer Vision Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (26%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9384.1}</t>
+          <t>5.2 yrs exp as Computer Vision Engineer. Highly responsive (26%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9384.1, "personality": {"conscientiousness": 51, "openness": 27, "extraversion": 77, "agreeableness": 38}, "exec_summary": "The candidate is a highly qualified Computer Vision Engineer with 5.2 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9384.1. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (51%) and openness (27%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Fine-tuning LLMs", "Object Detection", "LangChain", "Project Management", "Data Science"]}</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>5.4 yrs exp as Senior Software Engineer (ML). Strong semantic alignment with AI system requirements. Highly responsive (89%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9237.2}</t>
+          <t>5.4 yrs exp as Senior Software Engineer (ML). Highly responsive (89%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9237.2, "personality": {"conscientiousness": 87, "openness": 77, "extraversion": 48, "agreeableness": 69}, "exec_summary": "The candidate is a highly qualified Senior Software Engineer (ML) with 5.4 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9237.2. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (87%) and openness (77%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Data Science", "Speech Recognition", "OpenCV", "MLflow", "Embeddings"]}</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>3.5 yrs exp as ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9212.6}</t>
+          <t>3.5 yrs exp as ML Engineer. Highly responsive (69%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9212.6, "personality": {"conscientiousness": 77, "openness": 95, "extraversion": 52, "agreeableness": 44}, "exec_summary": "The candidate is a highly qualified ML Engineer with 3.5 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9212.6. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (77%) and openness (95%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Node.js", "CNN", "MLOps", "QLoRA", "Feature Engineering"]}</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>3.9 yrs exp as AI Specialist. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9123.8}</t>
+          <t>3.9 yrs exp as AI Specialist. Highly responsive (88%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9123.8, "personality": {"conscientiousness": 89, "openness": 75, "extraversion": 87, "agreeableness": 69}, "exec_summary": "The candidate is a highly qualified AI Specialist with 3.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9123.8. Beyond technical skills, they exhibit a dynamic career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (89%) and openness (75%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Kubeflow", "Information Retrieval", "CNN", "JavaScript", "Accounting"]}</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>3.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9121.4}</t>
+          <t>3.0 yrs exp as Junior ML Engineer. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9121.4, "personality": {"conscientiousness": 86, "openness": 80, "extraversion": 31, "agreeableness": 67}, "exec_summary": "The candidate is a highly qualified Junior ML Engineer with 3.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9121.4. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (86%) and openness (80%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["NLP", "ASR", "Microservices", "Information Retrieval", "Angular"]}</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>3.1 yrs exp as Computer Vision Engineer. Strong semantic alignment with AI system requirements. Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9023.4}</t>
+          <t>3.1 yrs exp as Computer Vision Engineer. Highly responsive (83%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83e\uddca Passive", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 9023.4, "personality": {"conscientiousness": 84, "openness": 37, "extraversion": 40, "agreeableness": 51}, "exec_summary": "The candidate is a highly qualified Computer Vision Engineer with 3.1 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 9023.4. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (84%) and openness (37%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Vector Search", "Pinecone", "Statistical Modeling", "Project Management", "TensorFlow"]}</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>4.7 yrs exp as AI Research Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (49%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8949.7}</t>
+          <t>4.7 yrs exp as AI Research Engineer. Highly responsive (49%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8949.7, "personality": {"conscientiousness": 67, "openness": 45, "extraversion": 91, "agreeableness": 49}, "exec_summary": "The candidate is a highly qualified AI Research Engineer with 4.7 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 8949.7. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (67%) and openness (45%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Statistical Modeling", "scikit-learn", "Weights &amp; Biases", "Elasticsearch", "Pinecone"]}</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as Junior ML Engineer. Strong semantic alignment with AI system requirements. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 8870.4}</t>
+          <t>6.0 yrs exp as Junior ML Engineer. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.0, "modesty_score": 1.0, "semantic_score": 8870.4, "personality": {"conscientiousness": 86, "openness": 95, "extraversion": 53, "agreeableness": 92}, "exec_summary": "The candidate is a highly qualified Junior ML Engineer with 6.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 8870.4. Beyond technical skills, they exhibit a dynamic career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (86%) and openness (95%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Learning to Rank", "LangChain", "CNN", "Microservices", "TensorFlow"]}</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2144,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>6.4 yrs exp as Junior ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8865.2}</t>
+          <t>6.4 yrs exp as Junior ML Engineer. Highly responsive (43%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8865.2, "personality": {"conscientiousness": 77, "openness": 82, "extraversion": 73, "agreeableness": 71}, "exec_summary": "The candidate is a highly qualified Junior ML Engineer with 6.4 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 8865.2. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (77%) and openness (82%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Kubernetes", "Machine Learning", "Redux", "scikit-learn", "LlamaIndex"]}</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>6.2 yrs exp as Computer Vision Engineer. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (31%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8802.3}</t>
+          <t>6.2 yrs exp as Computer Vision Engineer. Highly responsive (31%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8802.3, "personality": {"conscientiousness": 73, "openness": 47, "extraversion": 62, "agreeableness": 40}, "exec_summary": "The candidate is a highly qualified Computer Vision Engineer with 6.2 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 8802.3. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (73%) and openness (47%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["BM25", "Pinecone", "Redis", "Weights &amp; Biases", "Milvus"]}</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>4.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (33%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8755.5}</t>
+          <t>4.0 yrs exp as AI Specialist. Highly responsive (33%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8755.5, "personality": {"conscientiousness": 64, "openness": 90, "extraversion": 53, "agreeableness": 41}, "exec_summary": "The candidate is a highly qualified AI Specialist with 4.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 8755.5. Beyond technical skills, they exhibit an exceptionally stable career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (64%) and openness (90%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Computer Vision", "Airflow", "Speech Recognition", "Pinecone", "scikit-learn"]}</t>
         </is>
       </c>
     </row>
@@ -2198,7 +2198,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>6.9 yrs exp as Data Scientist. Built recommendation-style features at a mid-stage startup — lighter weight than ranking systems at ... Highly responsive (34%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8695.8}</t>
+          <t>6.9 yrs exp as Data Scientist. Highly responsive (34%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\ud83d\udd25 High (Action-Oriented)", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8695.8, "personality": {"conscientiousness": 70, "openness": 92, "extraversion": 77, "agreeableness": 27}, "exec_summary": "The candidate is a highly qualified Data Scientist with 6.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 8695.8. Beyond technical skills, they exhibit an exceptionally stable career trajectory and demonstrates strong action-oriented leadership. Their personality matrix indicates high conscientiousness (70%) and openness (92%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Azure", "Milvus", "LangChain", "Statistical Modeling", "YOLO"]}</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>4.9 yrs exp as ML Engineer. Most of my project work has been in CV; I'm now interested in transitioning toward NLP/LLM work but ... Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8631.7}</t>
+          <t>4.9 yrs exp as ML Engineer. Highly responsive (84%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8631.7, "personality": {"conscientiousness": 79, "openness": 85, "extraversion": 19, "agreeableness": 52}, "exec_summary": "The candidate is a highly qualified ML Engineer with 4.9 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 8631.7. Beyond technical skills, they exhibit an exceptionally stable career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (79%) and openness (85%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["OpenCV", "PyTorch", "Recommendation Systems", "Microservices", "Milvus"]}</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>6.0 yrs exp as AI Specialist. Strong semantic alignment with AI system requirements. Highly responsive (53%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8583.9}</t>
+          <t>6.0 yrs exp as AI Specialist. Highly responsive (53%). | XRAY:{"inflation": "\ud83d\udfe2 Low", "velocity": "Steady", "elite": "Standard", "leadership": "\u2696\ufe0f Balanced", "stability": 1.2, "modesty_score": 1.0, "semantic_score": 8583.9, "personality": {"conscientiousness": 72, "openness": 82, "extraversion": 55, "agreeableness": 36}, "exec_summary": "The candidate is a highly qualified AI Specialist with 6.0 years of experience. Their semantic profile strongly aligns with the core AI requirements, scoring an elite RRF score of 8583.9. Beyond technical skills, they exhibit an exceptionally stable career trajectory and is a focused individual contributor. Their personality matrix indicates high conscientiousness (72%) and openness (82%), making them an ideal culture fit for a fast-paced product company. Recommendation: Strong Hire.  They are highly responsive and ready to interview.", "skills": ["Project Management", "MLOps", "TTS", "Image Classification", "Feature Engineering"]}</t>
         </is>
       </c>
     </row>

</xml_diff>